<commit_message>
Add caution column to convoy spreadsheet
</commit_message>
<xml_diff>
--- a/convois_epr2.xlsx
+++ b/convois_epr2.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feuil1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feuil1'!$A$1:$J$501</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feuil1'!$A$1:$K$501</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Feuil1'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -158,9 +158,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TableConvoisEPR2" displayName="TableConvoisEPR2" ref="A1:J501" headerRowCount="1">
-  <autoFilter ref="A1:J501"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TableConvoisEPR2" displayName="TableConvoisEPR2" ref="A1:K501" headerRowCount="1">
+  <autoFilter ref="A1:K501"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="N°"/>
     <tableColumn id="2" name="Nom"/>
     <tableColumn id="3" name="type de navire"/>
@@ -170,7 +170,8 @@
     <tableColumn id="7" name="colis"/>
     <tableColumn id="8" name="type de colis"/>
     <tableColumn id="9" name="justification"/>
-    <tableColumn id="10" name="pdf"/>
+    <tableColumn id="10" name="soit prudent"/>
+    <tableColumn id="11" name="pdf"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -465,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J501"/>
+  <dimension ref="A1:K501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -477,7 +478,8 @@
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -528,6 +530,11 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>soit prudent</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>pdf</t>
         </is>
       </c>
@@ -543,6 +550,7 @@
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
@@ -555,6 +563,7 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n"/>
@@ -567,6 +576,7 @@
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n"/>
@@ -579,6 +589,7 @@
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
@@ -591,6 +602,7 @@
       <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
@@ -603,6 +615,7 @@
       <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
@@ -615,6 +628,7 @@
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
@@ -627,6 +641,7 @@
       <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
@@ -639,6 +654,7 @@
       <c r="H10" s="3" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
@@ -651,6 +667,7 @@
       <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
@@ -663,6 +680,7 @@
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -675,6 +693,7 @@
       <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
+      <c r="K13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -687,6 +706,7 @@
       <c r="H14" s="3" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -699,6 +719,7 @@
       <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
@@ -711,6 +732,7 @@
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -723,6 +745,7 @@
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
+      <c r="K17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
@@ -735,6 +758,7 @@
       <c r="H18" s="3" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
@@ -747,6 +771,7 @@
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
@@ -759,6 +784,7 @@
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
+      <c r="K20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
@@ -771,6 +797,7 @@
       <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
+      <c r="K21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n"/>
@@ -783,6 +810,7 @@
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
@@ -795,6 +823,7 @@
       <c r="H23" s="3" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
@@ -807,6 +836,7 @@
       <c r="H24" s="3" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
@@ -819,6 +849,7 @@
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
@@ -831,6 +862,7 @@
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
@@ -843,6 +875,7 @@
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
@@ -855,6 +888,7 @@
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
@@ -867,6 +901,7 @@
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
@@ -879,6 +914,7 @@
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
@@ -891,6 +927,7 @@
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
@@ -903,6 +940,7 @@
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
+      <c r="K32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
@@ -915,6 +953,7 @@
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
@@ -927,6 +966,7 @@
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
@@ -939,6 +979,7 @@
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
@@ -951,6 +992,7 @@
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
@@ -963,6 +1005,7 @@
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
@@ -975,6 +1018,7 @@
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
+      <c r="K38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
@@ -987,6 +1031,7 @@
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
+      <c r="K39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
@@ -999,6 +1044,7 @@
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
+      <c r="K40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
@@ -1011,6 +1057,7 @@
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="n"/>
       <c r="J41" s="3" t="n"/>
+      <c r="K41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
@@ -1023,6 +1070,7 @@
       <c r="H42" s="3" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="3" t="n"/>
+      <c r="K42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
@@ -1035,6 +1083,7 @@
       <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
@@ -1047,6 +1096,7 @@
       <c r="H44" s="3" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="3" t="n"/>
+      <c r="K44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
@@ -1059,6 +1109,7 @@
       <c r="H45" s="3" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="3" t="n"/>
+      <c r="K45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
@@ -1071,6 +1122,7 @@
       <c r="H46" s="3" t="n"/>
       <c r="I46" s="3" t="n"/>
       <c r="J46" s="3" t="n"/>
+      <c r="K46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
@@ -1083,6 +1135,7 @@
       <c r="H47" s="3" t="n"/>
       <c r="I47" s="3" t="n"/>
       <c r="J47" s="3" t="n"/>
+      <c r="K47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -1095,6 +1148,7 @@
       <c r="H48" s="3" t="n"/>
       <c r="I48" s="3" t="n"/>
       <c r="J48" s="3" t="n"/>
+      <c r="K48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
@@ -1107,6 +1161,7 @@
       <c r="H49" s="3" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="3" t="n"/>
+      <c r="K49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -1119,6 +1174,7 @@
       <c r="H50" s="3" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="3" t="n"/>
+      <c r="K50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -1131,6 +1187,7 @@
       <c r="H51" s="3" t="n"/>
       <c r="I51" s="3" t="n"/>
       <c r="J51" s="3" t="n"/>
+      <c r="K51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -1143,6 +1200,7 @@
       <c r="H52" s="3" t="n"/>
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="n"/>
+      <c r="K52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -1155,6 +1213,7 @@
       <c r="H53" s="3" t="n"/>
       <c r="I53" s="3" t="n"/>
       <c r="J53" s="3" t="n"/>
+      <c r="K53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -1167,6 +1226,7 @@
       <c r="H54" s="3" t="n"/>
       <c r="I54" s="3" t="n"/>
       <c r="J54" s="3" t="n"/>
+      <c r="K54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -1179,6 +1239,7 @@
       <c r="H55" s="3" t="n"/>
       <c r="I55" s="3" t="n"/>
       <c r="J55" s="3" t="n"/>
+      <c r="K55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -1191,6 +1252,7 @@
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="n"/>
       <c r="J56" s="3" t="n"/>
+      <c r="K56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -1203,6 +1265,7 @@
       <c r="H57" s="3" t="n"/>
       <c r="I57" s="3" t="n"/>
       <c r="J57" s="3" t="n"/>
+      <c r="K57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -1215,6 +1278,7 @@
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="n"/>
       <c r="J58" s="3" t="n"/>
+      <c r="K58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -1227,6 +1291,7 @@
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="3" t="n"/>
       <c r="J59" s="3" t="n"/>
+      <c r="K59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -1239,6 +1304,7 @@
       <c r="H60" s="3" t="n"/>
       <c r="I60" s="3" t="n"/>
       <c r="J60" s="3" t="n"/>
+      <c r="K60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
@@ -1251,6 +1317,7 @@
       <c r="H61" s="3" t="n"/>
       <c r="I61" s="3" t="n"/>
       <c r="J61" s="3" t="n"/>
+      <c r="K61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
@@ -1263,6 +1330,7 @@
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="n"/>
       <c r="J62" s="3" t="n"/>
+      <c r="K62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
@@ -1275,6 +1343,7 @@
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="n"/>
       <c r="J63" s="3" t="n"/>
+      <c r="K63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
@@ -1287,6 +1356,7 @@
       <c r="H64" s="3" t="n"/>
       <c r="I64" s="3" t="n"/>
       <c r="J64" s="3" t="n"/>
+      <c r="K64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
@@ -1299,6 +1369,7 @@
       <c r="H65" s="3" t="n"/>
       <c r="I65" s="3" t="n"/>
       <c r="J65" s="3" t="n"/>
+      <c r="K65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
@@ -1311,6 +1382,7 @@
       <c r="H66" s="3" t="n"/>
       <c r="I66" s="3" t="n"/>
       <c r="J66" s="3" t="n"/>
+      <c r="K66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
@@ -1323,6 +1395,7 @@
       <c r="H67" s="3" t="n"/>
       <c r="I67" s="3" t="n"/>
       <c r="J67" s="3" t="n"/>
+      <c r="K67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
@@ -1335,6 +1408,7 @@
       <c r="H68" s="3" t="n"/>
       <c r="I68" s="3" t="n"/>
       <c r="J68" s="3" t="n"/>
+      <c r="K68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
@@ -1347,6 +1421,7 @@
       <c r="H69" s="3" t="n"/>
       <c r="I69" s="3" t="n"/>
       <c r="J69" s="3" t="n"/>
+      <c r="K69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
@@ -1359,6 +1434,7 @@
       <c r="H70" s="3" t="n"/>
       <c r="I70" s="3" t="n"/>
       <c r="J70" s="3" t="n"/>
+      <c r="K70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
@@ -1371,6 +1447,7 @@
       <c r="H71" s="3" t="n"/>
       <c r="I71" s="3" t="n"/>
       <c r="J71" s="3" t="n"/>
+      <c r="K71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
@@ -1383,6 +1460,7 @@
       <c r="H72" s="3" t="n"/>
       <c r="I72" s="3" t="n"/>
       <c r="J72" s="3" t="n"/>
+      <c r="K72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
@@ -1395,6 +1473,7 @@
       <c r="H73" s="3" t="n"/>
       <c r="I73" s="3" t="n"/>
       <c r="J73" s="3" t="n"/>
+      <c r="K73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
@@ -1407,6 +1486,7 @@
       <c r="H74" s="3" t="n"/>
       <c r="I74" s="3" t="n"/>
       <c r="J74" s="3" t="n"/>
+      <c r="K74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
@@ -1419,6 +1499,7 @@
       <c r="H75" s="3" t="n"/>
       <c r="I75" s="3" t="n"/>
       <c r="J75" s="3" t="n"/>
+      <c r="K75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
@@ -1431,6 +1512,7 @@
       <c r="H76" s="3" t="n"/>
       <c r="I76" s="3" t="n"/>
       <c r="J76" s="3" t="n"/>
+      <c r="K76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
@@ -1443,6 +1525,7 @@
       <c r="H77" s="3" t="n"/>
       <c r="I77" s="3" t="n"/>
       <c r="J77" s="3" t="n"/>
+      <c r="K77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
@@ -1455,6 +1538,7 @@
       <c r="H78" s="3" t="n"/>
       <c r="I78" s="3" t="n"/>
       <c r="J78" s="3" t="n"/>
+      <c r="K78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
@@ -1467,6 +1551,7 @@
       <c r="H79" s="3" t="n"/>
       <c r="I79" s="3" t="n"/>
       <c r="J79" s="3" t="n"/>
+      <c r="K79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
@@ -1479,6 +1564,7 @@
       <c r="H80" s="3" t="n"/>
       <c r="I80" s="3" t="n"/>
       <c r="J80" s="3" t="n"/>
+      <c r="K80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
@@ -1491,6 +1577,7 @@
       <c r="H81" s="3" t="n"/>
       <c r="I81" s="3" t="n"/>
       <c r="J81" s="3" t="n"/>
+      <c r="K81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
@@ -1503,6 +1590,7 @@
       <c r="H82" s="3" t="n"/>
       <c r="I82" s="3" t="n"/>
       <c r="J82" s="3" t="n"/>
+      <c r="K82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
@@ -1515,6 +1603,7 @@
       <c r="H83" s="3" t="n"/>
       <c r="I83" s="3" t="n"/>
       <c r="J83" s="3" t="n"/>
+      <c r="K83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
@@ -1527,6 +1616,7 @@
       <c r="H84" s="3" t="n"/>
       <c r="I84" s="3" t="n"/>
       <c r="J84" s="3" t="n"/>
+      <c r="K84" s="3" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
@@ -1539,6 +1629,7 @@
       <c r="H85" s="3" t="n"/>
       <c r="I85" s="3" t="n"/>
       <c r="J85" s="3" t="n"/>
+      <c r="K85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
@@ -1551,6 +1642,7 @@
       <c r="H86" s="3" t="n"/>
       <c r="I86" s="3" t="n"/>
       <c r="J86" s="3" t="n"/>
+      <c r="K86" s="3" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
@@ -1563,6 +1655,7 @@
       <c r="H87" s="3" t="n"/>
       <c r="I87" s="3" t="n"/>
       <c r="J87" s="3" t="n"/>
+      <c r="K87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
@@ -1575,6 +1668,7 @@
       <c r="H88" s="3" t="n"/>
       <c r="I88" s="3" t="n"/>
       <c r="J88" s="3" t="n"/>
+      <c r="K88" s="3" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
@@ -1587,6 +1681,7 @@
       <c r="H89" s="3" t="n"/>
       <c r="I89" s="3" t="n"/>
       <c r="J89" s="3" t="n"/>
+      <c r="K89" s="3" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
@@ -1599,6 +1694,7 @@
       <c r="H90" s="3" t="n"/>
       <c r="I90" s="3" t="n"/>
       <c r="J90" s="3" t="n"/>
+      <c r="K90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
@@ -1611,6 +1707,7 @@
       <c r="H91" s="3" t="n"/>
       <c r="I91" s="3" t="n"/>
       <c r="J91" s="3" t="n"/>
+      <c r="K91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
@@ -1623,6 +1720,7 @@
       <c r="H92" s="3" t="n"/>
       <c r="I92" s="3" t="n"/>
       <c r="J92" s="3" t="n"/>
+      <c r="K92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
@@ -1635,6 +1733,7 @@
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3" t="n"/>
       <c r="J93" s="3" t="n"/>
+      <c r="K93" s="3" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
@@ -1647,6 +1746,7 @@
       <c r="H94" s="3" t="n"/>
       <c r="I94" s="3" t="n"/>
       <c r="J94" s="3" t="n"/>
+      <c r="K94" s="3" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
@@ -1659,6 +1759,7 @@
       <c r="H95" s="3" t="n"/>
       <c r="I95" s="3" t="n"/>
       <c r="J95" s="3" t="n"/>
+      <c r="K95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
@@ -1671,6 +1772,7 @@
       <c r="H96" s="3" t="n"/>
       <c r="I96" s="3" t="n"/>
       <c r="J96" s="3" t="n"/>
+      <c r="K96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n"/>
@@ -1683,6 +1785,7 @@
       <c r="H97" s="3" t="n"/>
       <c r="I97" s="3" t="n"/>
       <c r="J97" s="3" t="n"/>
+      <c r="K97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n"/>
@@ -1695,6 +1798,7 @@
       <c r="H98" s="3" t="n"/>
       <c r="I98" s="3" t="n"/>
       <c r="J98" s="3" t="n"/>
+      <c r="K98" s="3" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n"/>
@@ -1707,6 +1811,7 @@
       <c r="H99" s="3" t="n"/>
       <c r="I99" s="3" t="n"/>
       <c r="J99" s="3" t="n"/>
+      <c r="K99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n"/>
@@ -1719,6 +1824,7 @@
       <c r="H100" s="3" t="n"/>
       <c r="I100" s="3" t="n"/>
       <c r="J100" s="3" t="n"/>
+      <c r="K100" s="3" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n"/>
@@ -1731,6 +1837,7 @@
       <c r="H101" s="3" t="n"/>
       <c r="I101" s="3" t="n"/>
       <c r="J101" s="3" t="n"/>
+      <c r="K101" s="3" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n"/>
@@ -1743,6 +1850,7 @@
       <c r="H102" s="3" t="n"/>
       <c r="I102" s="3" t="n"/>
       <c r="J102" s="3" t="n"/>
+      <c r="K102" s="3" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n"/>
@@ -1755,6 +1863,7 @@
       <c r="H103" s="3" t="n"/>
       <c r="I103" s="3" t="n"/>
       <c r="J103" s="3" t="n"/>
+      <c r="K103" s="3" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n"/>
@@ -1767,6 +1876,7 @@
       <c r="H104" s="3" t="n"/>
       <c r="I104" s="3" t="n"/>
       <c r="J104" s="3" t="n"/>
+      <c r="K104" s="3" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n"/>
@@ -1779,6 +1889,7 @@
       <c r="H105" s="3" t="n"/>
       <c r="I105" s="3" t="n"/>
       <c r="J105" s="3" t="n"/>
+      <c r="K105" s="3" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n"/>
@@ -1791,6 +1902,7 @@
       <c r="H106" s="3" t="n"/>
       <c r="I106" s="3" t="n"/>
       <c r="J106" s="3" t="n"/>
+      <c r="K106" s="3" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n"/>
@@ -1803,6 +1915,7 @@
       <c r="H107" s="3" t="n"/>
       <c r="I107" s="3" t="n"/>
       <c r="J107" s="3" t="n"/>
+      <c r="K107" s="3" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n"/>
@@ -1815,6 +1928,7 @@
       <c r="H108" s="3" t="n"/>
       <c r="I108" s="3" t="n"/>
       <c r="J108" s="3" t="n"/>
+      <c r="K108" s="3" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n"/>
@@ -1827,6 +1941,7 @@
       <c r="H109" s="3" t="n"/>
       <c r="I109" s="3" t="n"/>
       <c r="J109" s="3" t="n"/>
+      <c r="K109" s="3" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n"/>
@@ -1839,6 +1954,7 @@
       <c r="H110" s="3" t="n"/>
       <c r="I110" s="3" t="n"/>
       <c r="J110" s="3" t="n"/>
+      <c r="K110" s="3" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n"/>
@@ -1851,6 +1967,7 @@
       <c r="H111" s="3" t="n"/>
       <c r="I111" s="3" t="n"/>
       <c r="J111" s="3" t="n"/>
+      <c r="K111" s="3" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n"/>
@@ -1863,6 +1980,7 @@
       <c r="H112" s="3" t="n"/>
       <c r="I112" s="3" t="n"/>
       <c r="J112" s="3" t="n"/>
+      <c r="K112" s="3" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n"/>
@@ -1875,6 +1993,7 @@
       <c r="H113" s="3" t="n"/>
       <c r="I113" s="3" t="n"/>
       <c r="J113" s="3" t="n"/>
+      <c r="K113" s="3" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n"/>
@@ -1887,6 +2006,7 @@
       <c r="H114" s="3" t="n"/>
       <c r="I114" s="3" t="n"/>
       <c r="J114" s="3" t="n"/>
+      <c r="K114" s="3" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n"/>
@@ -1899,6 +2019,7 @@
       <c r="H115" s="3" t="n"/>
       <c r="I115" s="3" t="n"/>
       <c r="J115" s="3" t="n"/>
+      <c r="K115" s="3" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n"/>
@@ -1911,6 +2032,7 @@
       <c r="H116" s="3" t="n"/>
       <c r="I116" s="3" t="n"/>
       <c r="J116" s="3" t="n"/>
+      <c r="K116" s="3" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n"/>
@@ -1923,6 +2045,7 @@
       <c r="H117" s="3" t="n"/>
       <c r="I117" s="3" t="n"/>
       <c r="J117" s="3" t="n"/>
+      <c r="K117" s="3" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n"/>
@@ -1935,6 +2058,7 @@
       <c r="H118" s="3" t="n"/>
       <c r="I118" s="3" t="n"/>
       <c r="J118" s="3" t="n"/>
+      <c r="K118" s="3" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n"/>
@@ -1947,6 +2071,7 @@
       <c r="H119" s="3" t="n"/>
       <c r="I119" s="3" t="n"/>
       <c r="J119" s="3" t="n"/>
+      <c r="K119" s="3" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n"/>
@@ -1959,6 +2084,7 @@
       <c r="H120" s="3" t="n"/>
       <c r="I120" s="3" t="n"/>
       <c r="J120" s="3" t="n"/>
+      <c r="K120" s="3" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n"/>
@@ -1971,6 +2097,7 @@
       <c r="H121" s="3" t="n"/>
       <c r="I121" s="3" t="n"/>
       <c r="J121" s="3" t="n"/>
+      <c r="K121" s="3" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n"/>
@@ -1983,6 +2110,7 @@
       <c r="H122" s="3" t="n"/>
       <c r="I122" s="3" t="n"/>
       <c r="J122" s="3" t="n"/>
+      <c r="K122" s="3" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n"/>
@@ -1995,6 +2123,7 @@
       <c r="H123" s="3" t="n"/>
       <c r="I123" s="3" t="n"/>
       <c r="J123" s="3" t="n"/>
+      <c r="K123" s="3" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n"/>
@@ -2007,6 +2136,7 @@
       <c r="H124" s="3" t="n"/>
       <c r="I124" s="3" t="n"/>
       <c r="J124" s="3" t="n"/>
+      <c r="K124" s="3" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n"/>
@@ -2019,6 +2149,7 @@
       <c r="H125" s="3" t="n"/>
       <c r="I125" s="3" t="n"/>
       <c r="J125" s="3" t="n"/>
+      <c r="K125" s="3" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n"/>
@@ -2031,6 +2162,7 @@
       <c r="H126" s="3" t="n"/>
       <c r="I126" s="3" t="n"/>
       <c r="J126" s="3" t="n"/>
+      <c r="K126" s="3" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n"/>
@@ -2043,6 +2175,7 @@
       <c r="H127" s="3" t="n"/>
       <c r="I127" s="3" t="n"/>
       <c r="J127" s="3" t="n"/>
+      <c r="K127" s="3" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n"/>
@@ -2055,6 +2188,7 @@
       <c r="H128" s="3" t="n"/>
       <c r="I128" s="3" t="n"/>
       <c r="J128" s="3" t="n"/>
+      <c r="K128" s="3" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n"/>
@@ -2067,6 +2201,7 @@
       <c r="H129" s="3" t="n"/>
       <c r="I129" s="3" t="n"/>
       <c r="J129" s="3" t="n"/>
+      <c r="K129" s="3" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n"/>
@@ -2079,6 +2214,7 @@
       <c r="H130" s="3" t="n"/>
       <c r="I130" s="3" t="n"/>
       <c r="J130" s="3" t="n"/>
+      <c r="K130" s="3" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n"/>
@@ -2091,6 +2227,7 @@
       <c r="H131" s="3" t="n"/>
       <c r="I131" s="3" t="n"/>
       <c r="J131" s="3" t="n"/>
+      <c r="K131" s="3" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n"/>
@@ -2103,6 +2240,7 @@
       <c r="H132" s="3" t="n"/>
       <c r="I132" s="3" t="n"/>
       <c r="J132" s="3" t="n"/>
+      <c r="K132" s="3" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n"/>
@@ -2115,6 +2253,7 @@
       <c r="H133" s="3" t="n"/>
       <c r="I133" s="3" t="n"/>
       <c r="J133" s="3" t="n"/>
+      <c r="K133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n"/>
@@ -2127,6 +2266,7 @@
       <c r="H134" s="3" t="n"/>
       <c r="I134" s="3" t="n"/>
       <c r="J134" s="3" t="n"/>
+      <c r="K134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n"/>
@@ -2139,6 +2279,7 @@
       <c r="H135" s="3" t="n"/>
       <c r="I135" s="3" t="n"/>
       <c r="J135" s="3" t="n"/>
+      <c r="K135" s="3" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n"/>
@@ -2151,6 +2292,7 @@
       <c r="H136" s="3" t="n"/>
       <c r="I136" s="3" t="n"/>
       <c r="J136" s="3" t="n"/>
+      <c r="K136" s="3" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n"/>
@@ -2163,6 +2305,7 @@
       <c r="H137" s="3" t="n"/>
       <c r="I137" s="3" t="n"/>
       <c r="J137" s="3" t="n"/>
+      <c r="K137" s="3" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n"/>
@@ -2175,6 +2318,7 @@
       <c r="H138" s="3" t="n"/>
       <c r="I138" s="3" t="n"/>
       <c r="J138" s="3" t="n"/>
+      <c r="K138" s="3" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n"/>
@@ -2187,6 +2331,7 @@
       <c r="H139" s="3" t="n"/>
       <c r="I139" s="3" t="n"/>
       <c r="J139" s="3" t="n"/>
+      <c r="K139" s="3" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n"/>
@@ -2199,6 +2344,7 @@
       <c r="H140" s="3" t="n"/>
       <c r="I140" s="3" t="n"/>
       <c r="J140" s="3" t="n"/>
+      <c r="K140" s="3" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n"/>
@@ -2211,6 +2357,7 @@
       <c r="H141" s="3" t="n"/>
       <c r="I141" s="3" t="n"/>
       <c r="J141" s="3" t="n"/>
+      <c r="K141" s="3" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n"/>
@@ -2223,6 +2370,7 @@
       <c r="H142" s="3" t="n"/>
       <c r="I142" s="3" t="n"/>
       <c r="J142" s="3" t="n"/>
+      <c r="K142" s="3" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n"/>
@@ -2235,6 +2383,7 @@
       <c r="H143" s="3" t="n"/>
       <c r="I143" s="3" t="n"/>
       <c r="J143" s="3" t="n"/>
+      <c r="K143" s="3" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n"/>
@@ -2247,6 +2396,7 @@
       <c r="H144" s="3" t="n"/>
       <c r="I144" s="3" t="n"/>
       <c r="J144" s="3" t="n"/>
+      <c r="K144" s="3" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n"/>
@@ -2259,6 +2409,7 @@
       <c r="H145" s="3" t="n"/>
       <c r="I145" s="3" t="n"/>
       <c r="J145" s="3" t="n"/>
+      <c r="K145" s="3" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n"/>
@@ -2271,6 +2422,7 @@
       <c r="H146" s="3" t="n"/>
       <c r="I146" s="3" t="n"/>
       <c r="J146" s="3" t="n"/>
+      <c r="K146" s="3" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n"/>
@@ -2283,6 +2435,7 @@
       <c r="H147" s="3" t="n"/>
       <c r="I147" s="3" t="n"/>
       <c r="J147" s="3" t="n"/>
+      <c r="K147" s="3" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n"/>
@@ -2295,6 +2448,7 @@
       <c r="H148" s="3" t="n"/>
       <c r="I148" s="3" t="n"/>
       <c r="J148" s="3" t="n"/>
+      <c r="K148" s="3" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n"/>
@@ -2307,6 +2461,7 @@
       <c r="H149" s="3" t="n"/>
       <c r="I149" s="3" t="n"/>
       <c r="J149" s="3" t="n"/>
+      <c r="K149" s="3" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n"/>
@@ -2319,6 +2474,7 @@
       <c r="H150" s="3" t="n"/>
       <c r="I150" s="3" t="n"/>
       <c r="J150" s="3" t="n"/>
+      <c r="K150" s="3" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n"/>
@@ -2331,6 +2487,7 @@
       <c r="H151" s="3" t="n"/>
       <c r="I151" s="3" t="n"/>
       <c r="J151" s="3" t="n"/>
+      <c r="K151" s="3" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n"/>
@@ -2343,6 +2500,7 @@
       <c r="H152" s="3" t="n"/>
       <c r="I152" s="3" t="n"/>
       <c r="J152" s="3" t="n"/>
+      <c r="K152" s="3" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n"/>
@@ -2355,6 +2513,7 @@
       <c r="H153" s="3" t="n"/>
       <c r="I153" s="3" t="n"/>
       <c r="J153" s="3" t="n"/>
+      <c r="K153" s="3" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n"/>
@@ -2367,6 +2526,7 @@
       <c r="H154" s="3" t="n"/>
       <c r="I154" s="3" t="n"/>
       <c r="J154" s="3" t="n"/>
+      <c r="K154" s="3" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n"/>
@@ -2379,6 +2539,7 @@
       <c r="H155" s="3" t="n"/>
       <c r="I155" s="3" t="n"/>
       <c r="J155" s="3" t="n"/>
+      <c r="K155" s="3" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n"/>
@@ -2391,6 +2552,7 @@
       <c r="H156" s="3" t="n"/>
       <c r="I156" s="3" t="n"/>
       <c r="J156" s="3" t="n"/>
+      <c r="K156" s="3" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n"/>
@@ -2403,6 +2565,7 @@
       <c r="H157" s="3" t="n"/>
       <c r="I157" s="3" t="n"/>
       <c r="J157" s="3" t="n"/>
+      <c r="K157" s="3" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n"/>
@@ -2415,6 +2578,7 @@
       <c r="H158" s="3" t="n"/>
       <c r="I158" s="3" t="n"/>
       <c r="J158" s="3" t="n"/>
+      <c r="K158" s="3" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n"/>
@@ -2427,6 +2591,7 @@
       <c r="H159" s="3" t="n"/>
       <c r="I159" s="3" t="n"/>
       <c r="J159" s="3" t="n"/>
+      <c r="K159" s="3" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n"/>
@@ -2439,6 +2604,7 @@
       <c r="H160" s="3" t="n"/>
       <c r="I160" s="3" t="n"/>
       <c r="J160" s="3" t="n"/>
+      <c r="K160" s="3" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n"/>
@@ -2451,6 +2617,7 @@
       <c r="H161" s="3" t="n"/>
       <c r="I161" s="3" t="n"/>
       <c r="J161" s="3" t="n"/>
+      <c r="K161" s="3" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n"/>
@@ -2463,6 +2630,7 @@
       <c r="H162" s="3" t="n"/>
       <c r="I162" s="3" t="n"/>
       <c r="J162" s="3" t="n"/>
+      <c r="K162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n"/>
@@ -2475,6 +2643,7 @@
       <c r="H163" s="3" t="n"/>
       <c r="I163" s="3" t="n"/>
       <c r="J163" s="3" t="n"/>
+      <c r="K163" s="3" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n"/>
@@ -2487,6 +2656,7 @@
       <c r="H164" s="3" t="n"/>
       <c r="I164" s="3" t="n"/>
       <c r="J164" s="3" t="n"/>
+      <c r="K164" s="3" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n"/>
@@ -2499,6 +2669,7 @@
       <c r="H165" s="3" t="n"/>
       <c r="I165" s="3" t="n"/>
       <c r="J165" s="3" t="n"/>
+      <c r="K165" s="3" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n"/>
@@ -2511,6 +2682,7 @@
       <c r="H166" s="3" t="n"/>
       <c r="I166" s="3" t="n"/>
       <c r="J166" s="3" t="n"/>
+      <c r="K166" s="3" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n"/>
@@ -2523,6 +2695,7 @@
       <c r="H167" s="3" t="n"/>
       <c r="I167" s="3" t="n"/>
       <c r="J167" s="3" t="n"/>
+      <c r="K167" s="3" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n"/>
@@ -2535,6 +2708,7 @@
       <c r="H168" s="3" t="n"/>
       <c r="I168" s="3" t="n"/>
       <c r="J168" s="3" t="n"/>
+      <c r="K168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n"/>
@@ -2547,6 +2721,7 @@
       <c r="H169" s="3" t="n"/>
       <c r="I169" s="3" t="n"/>
       <c r="J169" s="3" t="n"/>
+      <c r="K169" s="3" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n"/>
@@ -2559,6 +2734,7 @@
       <c r="H170" s="3" t="n"/>
       <c r="I170" s="3" t="n"/>
       <c r="J170" s="3" t="n"/>
+      <c r="K170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n"/>
@@ -2571,6 +2747,7 @@
       <c r="H171" s="3" t="n"/>
       <c r="I171" s="3" t="n"/>
       <c r="J171" s="3" t="n"/>
+      <c r="K171" s="3" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n"/>
@@ -2583,6 +2760,7 @@
       <c r="H172" s="3" t="n"/>
       <c r="I172" s="3" t="n"/>
       <c r="J172" s="3" t="n"/>
+      <c r="K172" s="3" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n"/>
@@ -2595,6 +2773,7 @@
       <c r="H173" s="3" t="n"/>
       <c r="I173" s="3" t="n"/>
       <c r="J173" s="3" t="n"/>
+      <c r="K173" s="3" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n"/>
@@ -2607,6 +2786,7 @@
       <c r="H174" s="3" t="n"/>
       <c r="I174" s="3" t="n"/>
       <c r="J174" s="3" t="n"/>
+      <c r="K174" s="3" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n"/>
@@ -2619,6 +2799,7 @@
       <c r="H175" s="3" t="n"/>
       <c r="I175" s="3" t="n"/>
       <c r="J175" s="3" t="n"/>
+      <c r="K175" s="3" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n"/>
@@ -2631,6 +2812,7 @@
       <c r="H176" s="3" t="n"/>
       <c r="I176" s="3" t="n"/>
       <c r="J176" s="3" t="n"/>
+      <c r="K176" s="3" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n"/>
@@ -2643,6 +2825,7 @@
       <c r="H177" s="3" t="n"/>
       <c r="I177" s="3" t="n"/>
       <c r="J177" s="3" t="n"/>
+      <c r="K177" s="3" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n"/>
@@ -2655,6 +2838,7 @@
       <c r="H178" s="3" t="n"/>
       <c r="I178" s="3" t="n"/>
       <c r="J178" s="3" t="n"/>
+      <c r="K178" s="3" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n"/>
@@ -2667,6 +2851,7 @@
       <c r="H179" s="3" t="n"/>
       <c r="I179" s="3" t="n"/>
       <c r="J179" s="3" t="n"/>
+      <c r="K179" s="3" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n"/>
@@ -2679,6 +2864,7 @@
       <c r="H180" s="3" t="n"/>
       <c r="I180" s="3" t="n"/>
       <c r="J180" s="3" t="n"/>
+      <c r="K180" s="3" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n"/>
@@ -2691,6 +2877,7 @@
       <c r="H181" s="3" t="n"/>
       <c r="I181" s="3" t="n"/>
       <c r="J181" s="3" t="n"/>
+      <c r="K181" s="3" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n"/>
@@ -2703,6 +2890,7 @@
       <c r="H182" s="3" t="n"/>
       <c r="I182" s="3" t="n"/>
       <c r="J182" s="3" t="n"/>
+      <c r="K182" s="3" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n"/>
@@ -2715,6 +2903,7 @@
       <c r="H183" s="3" t="n"/>
       <c r="I183" s="3" t="n"/>
       <c r="J183" s="3" t="n"/>
+      <c r="K183" s="3" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n"/>
@@ -2727,6 +2916,7 @@
       <c r="H184" s="3" t="n"/>
       <c r="I184" s="3" t="n"/>
       <c r="J184" s="3" t="n"/>
+      <c r="K184" s="3" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n"/>
@@ -2739,6 +2929,7 @@
       <c r="H185" s="3" t="n"/>
       <c r="I185" s="3" t="n"/>
       <c r="J185" s="3" t="n"/>
+      <c r="K185" s="3" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n"/>
@@ -2751,6 +2942,7 @@
       <c r="H186" s="3" t="n"/>
       <c r="I186" s="3" t="n"/>
       <c r="J186" s="3" t="n"/>
+      <c r="K186" s="3" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n"/>
@@ -2763,6 +2955,7 @@
       <c r="H187" s="3" t="n"/>
       <c r="I187" s="3" t="n"/>
       <c r="J187" s="3" t="n"/>
+      <c r="K187" s="3" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n"/>
@@ -2775,6 +2968,7 @@
       <c r="H188" s="3" t="n"/>
       <c r="I188" s="3" t="n"/>
       <c r="J188" s="3" t="n"/>
+      <c r="K188" s="3" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n"/>
@@ -2787,6 +2981,7 @@
       <c r="H189" s="3" t="n"/>
       <c r="I189" s="3" t="n"/>
       <c r="J189" s="3" t="n"/>
+      <c r="K189" s="3" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n"/>
@@ -2799,6 +2994,7 @@
       <c r="H190" s="3" t="n"/>
       <c r="I190" s="3" t="n"/>
       <c r="J190" s="3" t="n"/>
+      <c r="K190" s="3" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n"/>
@@ -2811,6 +3007,7 @@
       <c r="H191" s="3" t="n"/>
       <c r="I191" s="3" t="n"/>
       <c r="J191" s="3" t="n"/>
+      <c r="K191" s="3" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n"/>
@@ -2823,6 +3020,7 @@
       <c r="H192" s="3" t="n"/>
       <c r="I192" s="3" t="n"/>
       <c r="J192" s="3" t="n"/>
+      <c r="K192" s="3" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n"/>
@@ -2835,6 +3033,7 @@
       <c r="H193" s="3" t="n"/>
       <c r="I193" s="3" t="n"/>
       <c r="J193" s="3" t="n"/>
+      <c r="K193" s="3" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n"/>
@@ -2847,6 +3046,7 @@
       <c r="H194" s="3" t="n"/>
       <c r="I194" s="3" t="n"/>
       <c r="J194" s="3" t="n"/>
+      <c r="K194" s="3" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n"/>
@@ -2859,6 +3059,7 @@
       <c r="H195" s="3" t="n"/>
       <c r="I195" s="3" t="n"/>
       <c r="J195" s="3" t="n"/>
+      <c r="K195" s="3" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n"/>
@@ -2871,6 +3072,7 @@
       <c r="H196" s="3" t="n"/>
       <c r="I196" s="3" t="n"/>
       <c r="J196" s="3" t="n"/>
+      <c r="K196" s="3" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n"/>
@@ -2883,6 +3085,7 @@
       <c r="H197" s="3" t="n"/>
       <c r="I197" s="3" t="n"/>
       <c r="J197" s="3" t="n"/>
+      <c r="K197" s="3" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n"/>
@@ -2895,6 +3098,7 @@
       <c r="H198" s="3" t="n"/>
       <c r="I198" s="3" t="n"/>
       <c r="J198" s="3" t="n"/>
+      <c r="K198" s="3" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n"/>
@@ -2907,6 +3111,7 @@
       <c r="H199" s="3" t="n"/>
       <c r="I199" s="3" t="n"/>
       <c r="J199" s="3" t="n"/>
+      <c r="K199" s="3" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n"/>
@@ -2919,6 +3124,7 @@
       <c r="H200" s="3" t="n"/>
       <c r="I200" s="3" t="n"/>
       <c r="J200" s="3" t="n"/>
+      <c r="K200" s="3" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n"/>
@@ -2931,6 +3137,7 @@
       <c r="H201" s="3" t="n"/>
       <c r="I201" s="3" t="n"/>
       <c r="J201" s="3" t="n"/>
+      <c r="K201" s="3" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n"/>
@@ -2943,6 +3150,7 @@
       <c r="H202" s="3" t="n"/>
       <c r="I202" s="3" t="n"/>
       <c r="J202" s="3" t="n"/>
+      <c r="K202" s="3" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n"/>
@@ -2955,6 +3163,7 @@
       <c r="H203" s="3" t="n"/>
       <c r="I203" s="3" t="n"/>
       <c r="J203" s="3" t="n"/>
+      <c r="K203" s="3" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n"/>
@@ -2967,6 +3176,7 @@
       <c r="H204" s="3" t="n"/>
       <c r="I204" s="3" t="n"/>
       <c r="J204" s="3" t="n"/>
+      <c r="K204" s="3" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n"/>
@@ -2979,6 +3189,7 @@
       <c r="H205" s="3" t="n"/>
       <c r="I205" s="3" t="n"/>
       <c r="J205" s="3" t="n"/>
+      <c r="K205" s="3" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n"/>
@@ -2991,6 +3202,7 @@
       <c r="H206" s="3" t="n"/>
       <c r="I206" s="3" t="n"/>
       <c r="J206" s="3" t="n"/>
+      <c r="K206" s="3" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n"/>
@@ -3003,6 +3215,7 @@
       <c r="H207" s="3" t="n"/>
       <c r="I207" s="3" t="n"/>
       <c r="J207" s="3" t="n"/>
+      <c r="K207" s="3" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n"/>
@@ -3015,6 +3228,7 @@
       <c r="H208" s="3" t="n"/>
       <c r="I208" s="3" t="n"/>
       <c r="J208" s="3" t="n"/>
+      <c r="K208" s="3" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n"/>
@@ -3027,6 +3241,7 @@
       <c r="H209" s="3" t="n"/>
       <c r="I209" s="3" t="n"/>
       <c r="J209" s="3" t="n"/>
+      <c r="K209" s="3" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n"/>
@@ -3039,6 +3254,7 @@
       <c r="H210" s="3" t="n"/>
       <c r="I210" s="3" t="n"/>
       <c r="J210" s="3" t="n"/>
+      <c r="K210" s="3" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n"/>
@@ -3051,6 +3267,7 @@
       <c r="H211" s="3" t="n"/>
       <c r="I211" s="3" t="n"/>
       <c r="J211" s="3" t="n"/>
+      <c r="K211" s="3" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n"/>
@@ -3063,6 +3280,7 @@
       <c r="H212" s="3" t="n"/>
       <c r="I212" s="3" t="n"/>
       <c r="J212" s="3" t="n"/>
+      <c r="K212" s="3" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n"/>
@@ -3075,6 +3293,7 @@
       <c r="H213" s="3" t="n"/>
       <c r="I213" s="3" t="n"/>
       <c r="J213" s="3" t="n"/>
+      <c r="K213" s="3" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n"/>
@@ -3087,6 +3306,7 @@
       <c r="H214" s="3" t="n"/>
       <c r="I214" s="3" t="n"/>
       <c r="J214" s="3" t="n"/>
+      <c r="K214" s="3" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n"/>
@@ -3099,6 +3319,7 @@
       <c r="H215" s="3" t="n"/>
       <c r="I215" s="3" t="n"/>
       <c r="J215" s="3" t="n"/>
+      <c r="K215" s="3" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n"/>
@@ -3111,6 +3332,7 @@
       <c r="H216" s="3" t="n"/>
       <c r="I216" s="3" t="n"/>
       <c r="J216" s="3" t="n"/>
+      <c r="K216" s="3" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n"/>
@@ -3123,6 +3345,7 @@
       <c r="H217" s="3" t="n"/>
       <c r="I217" s="3" t="n"/>
       <c r="J217" s="3" t="n"/>
+      <c r="K217" s="3" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n"/>
@@ -3135,6 +3358,7 @@
       <c r="H218" s="3" t="n"/>
       <c r="I218" s="3" t="n"/>
       <c r="J218" s="3" t="n"/>
+      <c r="K218" s="3" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n"/>
@@ -3147,6 +3371,7 @@
       <c r="H219" s="3" t="n"/>
       <c r="I219" s="3" t="n"/>
       <c r="J219" s="3" t="n"/>
+      <c r="K219" s="3" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n"/>
@@ -3159,6 +3384,7 @@
       <c r="H220" s="3" t="n"/>
       <c r="I220" s="3" t="n"/>
       <c r="J220" s="3" t="n"/>
+      <c r="K220" s="3" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n"/>
@@ -3171,6 +3397,7 @@
       <c r="H221" s="3" t="n"/>
       <c r="I221" s="3" t="n"/>
       <c r="J221" s="3" t="n"/>
+      <c r="K221" s="3" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n"/>
@@ -3183,6 +3410,7 @@
       <c r="H222" s="3" t="n"/>
       <c r="I222" s="3" t="n"/>
       <c r="J222" s="3" t="n"/>
+      <c r="K222" s="3" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n"/>
@@ -3195,6 +3423,7 @@
       <c r="H223" s="3" t="n"/>
       <c r="I223" s="3" t="n"/>
       <c r="J223" s="3" t="n"/>
+      <c r="K223" s="3" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n"/>
@@ -3207,6 +3436,7 @@
       <c r="H224" s="3" t="n"/>
       <c r="I224" s="3" t="n"/>
       <c r="J224" s="3" t="n"/>
+      <c r="K224" s="3" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n"/>
@@ -3219,6 +3449,7 @@
       <c r="H225" s="3" t="n"/>
       <c r="I225" s="3" t="n"/>
       <c r="J225" s="3" t="n"/>
+      <c r="K225" s="3" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n"/>
@@ -3231,6 +3462,7 @@
       <c r="H226" s="3" t="n"/>
       <c r="I226" s="3" t="n"/>
       <c r="J226" s="3" t="n"/>
+      <c r="K226" s="3" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n"/>
@@ -3243,6 +3475,7 @@
       <c r="H227" s="3" t="n"/>
       <c r="I227" s="3" t="n"/>
       <c r="J227" s="3" t="n"/>
+      <c r="K227" s="3" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n"/>
@@ -3255,6 +3488,7 @@
       <c r="H228" s="3" t="n"/>
       <c r="I228" s="3" t="n"/>
       <c r="J228" s="3" t="n"/>
+      <c r="K228" s="3" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n"/>
@@ -3267,6 +3501,7 @@
       <c r="H229" s="3" t="n"/>
       <c r="I229" s="3" t="n"/>
       <c r="J229" s="3" t="n"/>
+      <c r="K229" s="3" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n"/>
@@ -3279,6 +3514,7 @@
       <c r="H230" s="3" t="n"/>
       <c r="I230" s="3" t="n"/>
       <c r="J230" s="3" t="n"/>
+      <c r="K230" s="3" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n"/>
@@ -3291,6 +3527,7 @@
       <c r="H231" s="3" t="n"/>
       <c r="I231" s="3" t="n"/>
       <c r="J231" s="3" t="n"/>
+      <c r="K231" s="3" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n"/>
@@ -3303,6 +3540,7 @@
       <c r="H232" s="3" t="n"/>
       <c r="I232" s="3" t="n"/>
       <c r="J232" s="3" t="n"/>
+      <c r="K232" s="3" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n"/>
@@ -3315,6 +3553,7 @@
       <c r="H233" s="3" t="n"/>
       <c r="I233" s="3" t="n"/>
       <c r="J233" s="3" t="n"/>
+      <c r="K233" s="3" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n"/>
@@ -3327,6 +3566,7 @@
       <c r="H234" s="3" t="n"/>
       <c r="I234" s="3" t="n"/>
       <c r="J234" s="3" t="n"/>
+      <c r="K234" s="3" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n"/>
@@ -3339,6 +3579,7 @@
       <c r="H235" s="3" t="n"/>
       <c r="I235" s="3" t="n"/>
       <c r="J235" s="3" t="n"/>
+      <c r="K235" s="3" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n"/>
@@ -3351,6 +3592,7 @@
       <c r="H236" s="3" t="n"/>
       <c r="I236" s="3" t="n"/>
       <c r="J236" s="3" t="n"/>
+      <c r="K236" s="3" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n"/>
@@ -3363,6 +3605,7 @@
       <c r="H237" s="3" t="n"/>
       <c r="I237" s="3" t="n"/>
       <c r="J237" s="3" t="n"/>
+      <c r="K237" s="3" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n"/>
@@ -3375,6 +3618,7 @@
       <c r="H238" s="3" t="n"/>
       <c r="I238" s="3" t="n"/>
       <c r="J238" s="3" t="n"/>
+      <c r="K238" s="3" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n"/>
@@ -3387,6 +3631,7 @@
       <c r="H239" s="3" t="n"/>
       <c r="I239" s="3" t="n"/>
       <c r="J239" s="3" t="n"/>
+      <c r="K239" s="3" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="n"/>
@@ -3399,6 +3644,7 @@
       <c r="H240" s="3" t="n"/>
       <c r="I240" s="3" t="n"/>
       <c r="J240" s="3" t="n"/>
+      <c r="K240" s="3" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n"/>
@@ -3411,6 +3657,7 @@
       <c r="H241" s="3" t="n"/>
       <c r="I241" s="3" t="n"/>
       <c r="J241" s="3" t="n"/>
+      <c r="K241" s="3" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n"/>
@@ -3423,6 +3670,7 @@
       <c r="H242" s="3" t="n"/>
       <c r="I242" s="3" t="n"/>
       <c r="J242" s="3" t="n"/>
+      <c r="K242" s="3" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n"/>
@@ -3435,6 +3683,7 @@
       <c r="H243" s="3" t="n"/>
       <c r="I243" s="3" t="n"/>
       <c r="J243" s="3" t="n"/>
+      <c r="K243" s="3" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="n"/>
@@ -3447,6 +3696,7 @@
       <c r="H244" s="3" t="n"/>
       <c r="I244" s="3" t="n"/>
       <c r="J244" s="3" t="n"/>
+      <c r="K244" s="3" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n"/>
@@ -3459,6 +3709,7 @@
       <c r="H245" s="3" t="n"/>
       <c r="I245" s="3" t="n"/>
       <c r="J245" s="3" t="n"/>
+      <c r="K245" s="3" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n"/>
@@ -3471,6 +3722,7 @@
       <c r="H246" s="3" t="n"/>
       <c r="I246" s="3" t="n"/>
       <c r="J246" s="3" t="n"/>
+      <c r="K246" s="3" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n"/>
@@ -3483,6 +3735,7 @@
       <c r="H247" s="3" t="n"/>
       <c r="I247" s="3" t="n"/>
       <c r="J247" s="3" t="n"/>
+      <c r="K247" s="3" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="n"/>
@@ -3495,6 +3748,7 @@
       <c r="H248" s="3" t="n"/>
       <c r="I248" s="3" t="n"/>
       <c r="J248" s="3" t="n"/>
+      <c r="K248" s="3" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="n"/>
@@ -3507,6 +3761,7 @@
       <c r="H249" s="3" t="n"/>
       <c r="I249" s="3" t="n"/>
       <c r="J249" s="3" t="n"/>
+      <c r="K249" s="3" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="n"/>
@@ -3519,6 +3774,7 @@
       <c r="H250" s="3" t="n"/>
       <c r="I250" s="3" t="n"/>
       <c r="J250" s="3" t="n"/>
+      <c r="K250" s="3" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="2" t="n"/>
@@ -3531,6 +3787,7 @@
       <c r="H251" s="3" t="n"/>
       <c r="I251" s="3" t="n"/>
       <c r="J251" s="3" t="n"/>
+      <c r="K251" s="3" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="2" t="n"/>
@@ -3543,6 +3800,7 @@
       <c r="H252" s="3" t="n"/>
       <c r="I252" s="3" t="n"/>
       <c r="J252" s="3" t="n"/>
+      <c r="K252" s="3" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="n"/>
@@ -3555,6 +3813,7 @@
       <c r="H253" s="3" t="n"/>
       <c r="I253" s="3" t="n"/>
       <c r="J253" s="3" t="n"/>
+      <c r="K253" s="3" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="2" t="n"/>
@@ -3567,6 +3826,7 @@
       <c r="H254" s="3" t="n"/>
       <c r="I254" s="3" t="n"/>
       <c r="J254" s="3" t="n"/>
+      <c r="K254" s="3" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="2" t="n"/>
@@ -3579,6 +3839,7 @@
       <c r="H255" s="3" t="n"/>
       <c r="I255" s="3" t="n"/>
       <c r="J255" s="3" t="n"/>
+      <c r="K255" s="3" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="2" t="n"/>
@@ -3591,6 +3852,7 @@
       <c r="H256" s="3" t="n"/>
       <c r="I256" s="3" t="n"/>
       <c r="J256" s="3" t="n"/>
+      <c r="K256" s="3" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="n"/>
@@ -3603,6 +3865,7 @@
       <c r="H257" s="3" t="n"/>
       <c r="I257" s="3" t="n"/>
       <c r="J257" s="3" t="n"/>
+      <c r="K257" s="3" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="2" t="n"/>
@@ -3615,6 +3878,7 @@
       <c r="H258" s="3" t="n"/>
       <c r="I258" s="3" t="n"/>
       <c r="J258" s="3" t="n"/>
+      <c r="K258" s="3" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="2" t="n"/>
@@ -3627,6 +3891,7 @@
       <c r="H259" s="3" t="n"/>
       <c r="I259" s="3" t="n"/>
       <c r="J259" s="3" t="n"/>
+      <c r="K259" s="3" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="2" t="n"/>
@@ -3639,6 +3904,7 @@
       <c r="H260" s="3" t="n"/>
       <c r="I260" s="3" t="n"/>
       <c r="J260" s="3" t="n"/>
+      <c r="K260" s="3" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="2" t="n"/>
@@ -3651,6 +3917,7 @@
       <c r="H261" s="3" t="n"/>
       <c r="I261" s="3" t="n"/>
       <c r="J261" s="3" t="n"/>
+      <c r="K261" s="3" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="2" t="n"/>
@@ -3663,6 +3930,7 @@
       <c r="H262" s="3" t="n"/>
       <c r="I262" s="3" t="n"/>
       <c r="J262" s="3" t="n"/>
+      <c r="K262" s="3" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="2" t="n"/>
@@ -3675,6 +3943,7 @@
       <c r="H263" s="3" t="n"/>
       <c r="I263" s="3" t="n"/>
       <c r="J263" s="3" t="n"/>
+      <c r="K263" s="3" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="2" t="n"/>
@@ -3687,6 +3956,7 @@
       <c r="H264" s="3" t="n"/>
       <c r="I264" s="3" t="n"/>
       <c r="J264" s="3" t="n"/>
+      <c r="K264" s="3" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="2" t="n"/>
@@ -3699,6 +3969,7 @@
       <c r="H265" s="3" t="n"/>
       <c r="I265" s="3" t="n"/>
       <c r="J265" s="3" t="n"/>
+      <c r="K265" s="3" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="2" t="n"/>
@@ -3711,6 +3982,7 @@
       <c r="H266" s="3" t="n"/>
       <c r="I266" s="3" t="n"/>
       <c r="J266" s="3" t="n"/>
+      <c r="K266" s="3" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="2" t="n"/>
@@ -3723,6 +3995,7 @@
       <c r="H267" s="3" t="n"/>
       <c r="I267" s="3" t="n"/>
       <c r="J267" s="3" t="n"/>
+      <c r="K267" s="3" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="2" t="n"/>
@@ -3735,6 +4008,7 @@
       <c r="H268" s="3" t="n"/>
       <c r="I268" s="3" t="n"/>
       <c r="J268" s="3" t="n"/>
+      <c r="K268" s="3" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="2" t="n"/>
@@ -3747,6 +4021,7 @@
       <c r="H269" s="3" t="n"/>
       <c r="I269" s="3" t="n"/>
       <c r="J269" s="3" t="n"/>
+      <c r="K269" s="3" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="2" t="n"/>
@@ -3759,6 +4034,7 @@
       <c r="H270" s="3" t="n"/>
       <c r="I270" s="3" t="n"/>
       <c r="J270" s="3" t="n"/>
+      <c r="K270" s="3" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="2" t="n"/>
@@ -3771,6 +4047,7 @@
       <c r="H271" s="3" t="n"/>
       <c r="I271" s="3" t="n"/>
       <c r="J271" s="3" t="n"/>
+      <c r="K271" s="3" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="2" t="n"/>
@@ -3783,6 +4060,7 @@
       <c r="H272" s="3" t="n"/>
       <c r="I272" s="3" t="n"/>
       <c r="J272" s="3" t="n"/>
+      <c r="K272" s="3" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="n"/>
@@ -3795,6 +4073,7 @@
       <c r="H273" s="3" t="n"/>
       <c r="I273" s="3" t="n"/>
       <c r="J273" s="3" t="n"/>
+      <c r="K273" s="3" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="n"/>
@@ -3807,6 +4086,7 @@
       <c r="H274" s="3" t="n"/>
       <c r="I274" s="3" t="n"/>
       <c r="J274" s="3" t="n"/>
+      <c r="K274" s="3" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="2" t="n"/>
@@ -3819,6 +4099,7 @@
       <c r="H275" s="3" t="n"/>
       <c r="I275" s="3" t="n"/>
       <c r="J275" s="3" t="n"/>
+      <c r="K275" s="3" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="2" t="n"/>
@@ -3831,6 +4112,7 @@
       <c r="H276" s="3" t="n"/>
       <c r="I276" s="3" t="n"/>
       <c r="J276" s="3" t="n"/>
+      <c r="K276" s="3" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="2" t="n"/>
@@ -3843,6 +4125,7 @@
       <c r="H277" s="3" t="n"/>
       <c r="I277" s="3" t="n"/>
       <c r="J277" s="3" t="n"/>
+      <c r="K277" s="3" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="2" t="n"/>
@@ -3855,6 +4138,7 @@
       <c r="H278" s="3" t="n"/>
       <c r="I278" s="3" t="n"/>
       <c r="J278" s="3" t="n"/>
+      <c r="K278" s="3" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="2" t="n"/>
@@ -3867,6 +4151,7 @@
       <c r="H279" s="3" t="n"/>
       <c r="I279" s="3" t="n"/>
       <c r="J279" s="3" t="n"/>
+      <c r="K279" s="3" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="2" t="n"/>
@@ -3879,6 +4164,7 @@
       <c r="H280" s="3" t="n"/>
       <c r="I280" s="3" t="n"/>
       <c r="J280" s="3" t="n"/>
+      <c r="K280" s="3" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="2" t="n"/>
@@ -3891,6 +4177,7 @@
       <c r="H281" s="3" t="n"/>
       <c r="I281" s="3" t="n"/>
       <c r="J281" s="3" t="n"/>
+      <c r="K281" s="3" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="2" t="n"/>
@@ -3903,6 +4190,7 @@
       <c r="H282" s="3" t="n"/>
       <c r="I282" s="3" t="n"/>
       <c r="J282" s="3" t="n"/>
+      <c r="K282" s="3" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="2" t="n"/>
@@ -3915,6 +4203,7 @@
       <c r="H283" s="3" t="n"/>
       <c r="I283" s="3" t="n"/>
       <c r="J283" s="3" t="n"/>
+      <c r="K283" s="3" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="2" t="n"/>
@@ -3927,6 +4216,7 @@
       <c r="H284" s="3" t="n"/>
       <c r="I284" s="3" t="n"/>
       <c r="J284" s="3" t="n"/>
+      <c r="K284" s="3" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="n"/>
@@ -3939,6 +4229,7 @@
       <c r="H285" s="3" t="n"/>
       <c r="I285" s="3" t="n"/>
       <c r="J285" s="3" t="n"/>
+      <c r="K285" s="3" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="n"/>
@@ -3951,6 +4242,7 @@
       <c r="H286" s="3" t="n"/>
       <c r="I286" s="3" t="n"/>
       <c r="J286" s="3" t="n"/>
+      <c r="K286" s="3" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="2" t="n"/>
@@ -3963,6 +4255,7 @@
       <c r="H287" s="3" t="n"/>
       <c r="I287" s="3" t="n"/>
       <c r="J287" s="3" t="n"/>
+      <c r="K287" s="3" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="2" t="n"/>
@@ -3975,6 +4268,7 @@
       <c r="H288" s="3" t="n"/>
       <c r="I288" s="3" t="n"/>
       <c r="J288" s="3" t="n"/>
+      <c r="K288" s="3" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="2" t="n"/>
@@ -3987,6 +4281,7 @@
       <c r="H289" s="3" t="n"/>
       <c r="I289" s="3" t="n"/>
       <c r="J289" s="3" t="n"/>
+      <c r="K289" s="3" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="2" t="n"/>
@@ -3999,6 +4294,7 @@
       <c r="H290" s="3" t="n"/>
       <c r="I290" s="3" t="n"/>
       <c r="J290" s="3" t="n"/>
+      <c r="K290" s="3" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="2" t="n"/>
@@ -4011,6 +4307,7 @@
       <c r="H291" s="3" t="n"/>
       <c r="I291" s="3" t="n"/>
       <c r="J291" s="3" t="n"/>
+      <c r="K291" s="3" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="2" t="n"/>
@@ -4023,6 +4320,7 @@
       <c r="H292" s="3" t="n"/>
       <c r="I292" s="3" t="n"/>
       <c r="J292" s="3" t="n"/>
+      <c r="K292" s="3" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="2" t="n"/>
@@ -4035,6 +4333,7 @@
       <c r="H293" s="3" t="n"/>
       <c r="I293" s="3" t="n"/>
       <c r="J293" s="3" t="n"/>
+      <c r="K293" s="3" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="n"/>
@@ -4047,6 +4346,7 @@
       <c r="H294" s="3" t="n"/>
       <c r="I294" s="3" t="n"/>
       <c r="J294" s="3" t="n"/>
+      <c r="K294" s="3" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="2" t="n"/>
@@ -4059,6 +4359,7 @@
       <c r="H295" s="3" t="n"/>
       <c r="I295" s="3" t="n"/>
       <c r="J295" s="3" t="n"/>
+      <c r="K295" s="3" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="2" t="n"/>
@@ -4071,6 +4372,7 @@
       <c r="H296" s="3" t="n"/>
       <c r="I296" s="3" t="n"/>
       <c r="J296" s="3" t="n"/>
+      <c r="K296" s="3" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="2" t="n"/>
@@ -4083,6 +4385,7 @@
       <c r="H297" s="3" t="n"/>
       <c r="I297" s="3" t="n"/>
       <c r="J297" s="3" t="n"/>
+      <c r="K297" s="3" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="2" t="n"/>
@@ -4095,6 +4398,7 @@
       <c r="H298" s="3" t="n"/>
       <c r="I298" s="3" t="n"/>
       <c r="J298" s="3" t="n"/>
+      <c r="K298" s="3" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="2" t="n"/>
@@ -4107,6 +4411,7 @@
       <c r="H299" s="3" t="n"/>
       <c r="I299" s="3" t="n"/>
       <c r="J299" s="3" t="n"/>
+      <c r="K299" s="3" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="2" t="n"/>
@@ -4119,6 +4424,7 @@
       <c r="H300" s="3" t="n"/>
       <c r="I300" s="3" t="n"/>
       <c r="J300" s="3" t="n"/>
+      <c r="K300" s="3" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="2" t="n"/>
@@ -4131,6 +4437,7 @@
       <c r="H301" s="3" t="n"/>
       <c r="I301" s="3" t="n"/>
       <c r="J301" s="3" t="n"/>
+      <c r="K301" s="3" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="2" t="n"/>
@@ -4143,6 +4450,7 @@
       <c r="H302" s="3" t="n"/>
       <c r="I302" s="3" t="n"/>
       <c r="J302" s="3" t="n"/>
+      <c r="K302" s="3" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="2" t="n"/>
@@ -4155,6 +4463,7 @@
       <c r="H303" s="3" t="n"/>
       <c r="I303" s="3" t="n"/>
       <c r="J303" s="3" t="n"/>
+      <c r="K303" s="3" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="2" t="n"/>
@@ -4167,6 +4476,7 @@
       <c r="H304" s="3" t="n"/>
       <c r="I304" s="3" t="n"/>
       <c r="J304" s="3" t="n"/>
+      <c r="K304" s="3" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="2" t="n"/>
@@ -4179,6 +4489,7 @@
       <c r="H305" s="3" t="n"/>
       <c r="I305" s="3" t="n"/>
       <c r="J305" s="3" t="n"/>
+      <c r="K305" s="3" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="2" t="n"/>
@@ -4191,6 +4502,7 @@
       <c r="H306" s="3" t="n"/>
       <c r="I306" s="3" t="n"/>
       <c r="J306" s="3" t="n"/>
+      <c r="K306" s="3" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="2" t="n"/>
@@ -4203,6 +4515,7 @@
       <c r="H307" s="3" t="n"/>
       <c r="I307" s="3" t="n"/>
       <c r="J307" s="3" t="n"/>
+      <c r="K307" s="3" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="n"/>
@@ -4215,6 +4528,7 @@
       <c r="H308" s="3" t="n"/>
       <c r="I308" s="3" t="n"/>
       <c r="J308" s="3" t="n"/>
+      <c r="K308" s="3" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="2" t="n"/>
@@ -4227,6 +4541,7 @@
       <c r="H309" s="3" t="n"/>
       <c r="I309" s="3" t="n"/>
       <c r="J309" s="3" t="n"/>
+      <c r="K309" s="3" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="2" t="n"/>
@@ -4239,6 +4554,7 @@
       <c r="H310" s="3" t="n"/>
       <c r="I310" s="3" t="n"/>
       <c r="J310" s="3" t="n"/>
+      <c r="K310" s="3" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="2" t="n"/>
@@ -4251,6 +4567,7 @@
       <c r="H311" s="3" t="n"/>
       <c r="I311" s="3" t="n"/>
       <c r="J311" s="3" t="n"/>
+      <c r="K311" s="3" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="2" t="n"/>
@@ -4263,6 +4580,7 @@
       <c r="H312" s="3" t="n"/>
       <c r="I312" s="3" t="n"/>
       <c r="J312" s="3" t="n"/>
+      <c r="K312" s="3" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="2" t="n"/>
@@ -4275,6 +4593,7 @@
       <c r="H313" s="3" t="n"/>
       <c r="I313" s="3" t="n"/>
       <c r="J313" s="3" t="n"/>
+      <c r="K313" s="3" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="2" t="n"/>
@@ -4287,6 +4606,7 @@
       <c r="H314" s="3" t="n"/>
       <c r="I314" s="3" t="n"/>
       <c r="J314" s="3" t="n"/>
+      <c r="K314" s="3" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="2" t="n"/>
@@ -4299,6 +4619,7 @@
       <c r="H315" s="3" t="n"/>
       <c r="I315" s="3" t="n"/>
       <c r="J315" s="3" t="n"/>
+      <c r="K315" s="3" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="2" t="n"/>
@@ -4311,6 +4632,7 @@
       <c r="H316" s="3" t="n"/>
       <c r="I316" s="3" t="n"/>
       <c r="J316" s="3" t="n"/>
+      <c r="K316" s="3" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="2" t="n"/>
@@ -4323,6 +4645,7 @@
       <c r="H317" s="3" t="n"/>
       <c r="I317" s="3" t="n"/>
       <c r="J317" s="3" t="n"/>
+      <c r="K317" s="3" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="2" t="n"/>
@@ -4335,6 +4658,7 @@
       <c r="H318" s="3" t="n"/>
       <c r="I318" s="3" t="n"/>
       <c r="J318" s="3" t="n"/>
+      <c r="K318" s="3" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="2" t="n"/>
@@ -4347,6 +4671,7 @@
       <c r="H319" s="3" t="n"/>
       <c r="I319" s="3" t="n"/>
       <c r="J319" s="3" t="n"/>
+      <c r="K319" s="3" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="2" t="n"/>
@@ -4359,6 +4684,7 @@
       <c r="H320" s="3" t="n"/>
       <c r="I320" s="3" t="n"/>
       <c r="J320" s="3" t="n"/>
+      <c r="K320" s="3" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="2" t="n"/>
@@ -4371,6 +4697,7 @@
       <c r="H321" s="3" t="n"/>
       <c r="I321" s="3" t="n"/>
       <c r="J321" s="3" t="n"/>
+      <c r="K321" s="3" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="2" t="n"/>
@@ -4383,6 +4710,7 @@
       <c r="H322" s="3" t="n"/>
       <c r="I322" s="3" t="n"/>
       <c r="J322" s="3" t="n"/>
+      <c r="K322" s="3" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="2" t="n"/>
@@ -4395,6 +4723,7 @@
       <c r="H323" s="3" t="n"/>
       <c r="I323" s="3" t="n"/>
       <c r="J323" s="3" t="n"/>
+      <c r="K323" s="3" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="2" t="n"/>
@@ -4407,6 +4736,7 @@
       <c r="H324" s="3" t="n"/>
       <c r="I324" s="3" t="n"/>
       <c r="J324" s="3" t="n"/>
+      <c r="K324" s="3" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="2" t="n"/>
@@ -4419,6 +4749,7 @@
       <c r="H325" s="3" t="n"/>
       <c r="I325" s="3" t="n"/>
       <c r="J325" s="3" t="n"/>
+      <c r="K325" s="3" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="2" t="n"/>
@@ -4431,6 +4762,7 @@
       <c r="H326" s="3" t="n"/>
       <c r="I326" s="3" t="n"/>
       <c r="J326" s="3" t="n"/>
+      <c r="K326" s="3" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="2" t="n"/>
@@ -4443,6 +4775,7 @@
       <c r="H327" s="3" t="n"/>
       <c r="I327" s="3" t="n"/>
       <c r="J327" s="3" t="n"/>
+      <c r="K327" s="3" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="2" t="n"/>
@@ -4455,6 +4788,7 @@
       <c r="H328" s="3" t="n"/>
       <c r="I328" s="3" t="n"/>
       <c r="J328" s="3" t="n"/>
+      <c r="K328" s="3" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="2" t="n"/>
@@ -4467,6 +4801,7 @@
       <c r="H329" s="3" t="n"/>
       <c r="I329" s="3" t="n"/>
       <c r="J329" s="3" t="n"/>
+      <c r="K329" s="3" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="2" t="n"/>
@@ -4479,6 +4814,7 @@
       <c r="H330" s="3" t="n"/>
       <c r="I330" s="3" t="n"/>
       <c r="J330" s="3" t="n"/>
+      <c r="K330" s="3" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="2" t="n"/>
@@ -4491,6 +4827,7 @@
       <c r="H331" s="3" t="n"/>
       <c r="I331" s="3" t="n"/>
       <c r="J331" s="3" t="n"/>
+      <c r="K331" s="3" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="2" t="n"/>
@@ -4503,6 +4840,7 @@
       <c r="H332" s="3" t="n"/>
       <c r="I332" s="3" t="n"/>
       <c r="J332" s="3" t="n"/>
+      <c r="K332" s="3" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="2" t="n"/>
@@ -4515,6 +4853,7 @@
       <c r="H333" s="3" t="n"/>
       <c r="I333" s="3" t="n"/>
       <c r="J333" s="3" t="n"/>
+      <c r="K333" s="3" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="2" t="n"/>
@@ -4527,6 +4866,7 @@
       <c r="H334" s="3" t="n"/>
       <c r="I334" s="3" t="n"/>
       <c r="J334" s="3" t="n"/>
+      <c r="K334" s="3" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="2" t="n"/>
@@ -4539,6 +4879,7 @@
       <c r="H335" s="3" t="n"/>
       <c r="I335" s="3" t="n"/>
       <c r="J335" s="3" t="n"/>
+      <c r="K335" s="3" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="2" t="n"/>
@@ -4551,6 +4892,7 @@
       <c r="H336" s="3" t="n"/>
       <c r="I336" s="3" t="n"/>
       <c r="J336" s="3" t="n"/>
+      <c r="K336" s="3" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="2" t="n"/>
@@ -4563,6 +4905,7 @@
       <c r="H337" s="3" t="n"/>
       <c r="I337" s="3" t="n"/>
       <c r="J337" s="3" t="n"/>
+      <c r="K337" s="3" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="2" t="n"/>
@@ -4575,6 +4918,7 @@
       <c r="H338" s="3" t="n"/>
       <c r="I338" s="3" t="n"/>
       <c r="J338" s="3" t="n"/>
+      <c r="K338" s="3" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="2" t="n"/>
@@ -4587,6 +4931,7 @@
       <c r="H339" s="3" t="n"/>
       <c r="I339" s="3" t="n"/>
       <c r="J339" s="3" t="n"/>
+      <c r="K339" s="3" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="2" t="n"/>
@@ -4599,6 +4944,7 @@
       <c r="H340" s="3" t="n"/>
       <c r="I340" s="3" t="n"/>
       <c r="J340" s="3" t="n"/>
+      <c r="K340" s="3" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="2" t="n"/>
@@ -4611,6 +4957,7 @@
       <c r="H341" s="3" t="n"/>
       <c r="I341" s="3" t="n"/>
       <c r="J341" s="3" t="n"/>
+      <c r="K341" s="3" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="2" t="n"/>
@@ -4623,6 +4970,7 @@
       <c r="H342" s="3" t="n"/>
       <c r="I342" s="3" t="n"/>
       <c r="J342" s="3" t="n"/>
+      <c r="K342" s="3" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="2" t="n"/>
@@ -4635,6 +4983,7 @@
       <c r="H343" s="3" t="n"/>
       <c r="I343" s="3" t="n"/>
       <c r="J343" s="3" t="n"/>
+      <c r="K343" s="3" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="2" t="n"/>
@@ -4647,6 +4996,7 @@
       <c r="H344" s="3" t="n"/>
       <c r="I344" s="3" t="n"/>
       <c r="J344" s="3" t="n"/>
+      <c r="K344" s="3" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="2" t="n"/>
@@ -4659,6 +5009,7 @@
       <c r="H345" s="3" t="n"/>
       <c r="I345" s="3" t="n"/>
       <c r="J345" s="3" t="n"/>
+      <c r="K345" s="3" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="2" t="n"/>
@@ -4671,6 +5022,7 @@
       <c r="H346" s="3" t="n"/>
       <c r="I346" s="3" t="n"/>
       <c r="J346" s="3" t="n"/>
+      <c r="K346" s="3" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="2" t="n"/>
@@ -4683,6 +5035,7 @@
       <c r="H347" s="3" t="n"/>
       <c r="I347" s="3" t="n"/>
       <c r="J347" s="3" t="n"/>
+      <c r="K347" s="3" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="2" t="n"/>
@@ -4695,6 +5048,7 @@
       <c r="H348" s="3" t="n"/>
       <c r="I348" s="3" t="n"/>
       <c r="J348" s="3" t="n"/>
+      <c r="K348" s="3" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="2" t="n"/>
@@ -4707,6 +5061,7 @@
       <c r="H349" s="3" t="n"/>
       <c r="I349" s="3" t="n"/>
       <c r="J349" s="3" t="n"/>
+      <c r="K349" s="3" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="2" t="n"/>
@@ -4719,6 +5074,7 @@
       <c r="H350" s="3" t="n"/>
       <c r="I350" s="3" t="n"/>
       <c r="J350" s="3" t="n"/>
+      <c r="K350" s="3" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="2" t="n"/>
@@ -4731,6 +5087,7 @@
       <c r="H351" s="3" t="n"/>
       <c r="I351" s="3" t="n"/>
       <c r="J351" s="3" t="n"/>
+      <c r="K351" s="3" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="2" t="n"/>
@@ -4743,6 +5100,7 @@
       <c r="H352" s="3" t="n"/>
       <c r="I352" s="3" t="n"/>
       <c r="J352" s="3" t="n"/>
+      <c r="K352" s="3" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="2" t="n"/>
@@ -4755,6 +5113,7 @@
       <c r="H353" s="3" t="n"/>
       <c r="I353" s="3" t="n"/>
       <c r="J353" s="3" t="n"/>
+      <c r="K353" s="3" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="2" t="n"/>
@@ -4767,6 +5126,7 @@
       <c r="H354" s="3" t="n"/>
       <c r="I354" s="3" t="n"/>
       <c r="J354" s="3" t="n"/>
+      <c r="K354" s="3" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="2" t="n"/>
@@ -4779,6 +5139,7 @@
       <c r="H355" s="3" t="n"/>
       <c r="I355" s="3" t="n"/>
       <c r="J355" s="3" t="n"/>
+      <c r="K355" s="3" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="2" t="n"/>
@@ -4791,6 +5152,7 @@
       <c r="H356" s="3" t="n"/>
       <c r="I356" s="3" t="n"/>
       <c r="J356" s="3" t="n"/>
+      <c r="K356" s="3" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="2" t="n"/>
@@ -4803,6 +5165,7 @@
       <c r="H357" s="3" t="n"/>
       <c r="I357" s="3" t="n"/>
       <c r="J357" s="3" t="n"/>
+      <c r="K357" s="3" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="2" t="n"/>
@@ -4815,6 +5178,7 @@
       <c r="H358" s="3" t="n"/>
       <c r="I358" s="3" t="n"/>
       <c r="J358" s="3" t="n"/>
+      <c r="K358" s="3" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="2" t="n"/>
@@ -4827,6 +5191,7 @@
       <c r="H359" s="3" t="n"/>
       <c r="I359" s="3" t="n"/>
       <c r="J359" s="3" t="n"/>
+      <c r="K359" s="3" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="2" t="n"/>
@@ -4839,6 +5204,7 @@
       <c r="H360" s="3" t="n"/>
       <c r="I360" s="3" t="n"/>
       <c r="J360" s="3" t="n"/>
+      <c r="K360" s="3" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="2" t="n"/>
@@ -4851,6 +5217,7 @@
       <c r="H361" s="3" t="n"/>
       <c r="I361" s="3" t="n"/>
       <c r="J361" s="3" t="n"/>
+      <c r="K361" s="3" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="2" t="n"/>
@@ -4863,6 +5230,7 @@
       <c r="H362" s="3" t="n"/>
       <c r="I362" s="3" t="n"/>
       <c r="J362" s="3" t="n"/>
+      <c r="K362" s="3" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="2" t="n"/>
@@ -4875,6 +5243,7 @@
       <c r="H363" s="3" t="n"/>
       <c r="I363" s="3" t="n"/>
       <c r="J363" s="3" t="n"/>
+      <c r="K363" s="3" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="2" t="n"/>
@@ -4887,6 +5256,7 @@
       <c r="H364" s="3" t="n"/>
       <c r="I364" s="3" t="n"/>
       <c r="J364" s="3" t="n"/>
+      <c r="K364" s="3" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="2" t="n"/>
@@ -4899,6 +5269,7 @@
       <c r="H365" s="3" t="n"/>
       <c r="I365" s="3" t="n"/>
       <c r="J365" s="3" t="n"/>
+      <c r="K365" s="3" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="2" t="n"/>
@@ -4911,6 +5282,7 @@
       <c r="H366" s="3" t="n"/>
       <c r="I366" s="3" t="n"/>
       <c r="J366" s="3" t="n"/>
+      <c r="K366" s="3" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="2" t="n"/>
@@ -4923,6 +5295,7 @@
       <c r="H367" s="3" t="n"/>
       <c r="I367" s="3" t="n"/>
       <c r="J367" s="3" t="n"/>
+      <c r="K367" s="3" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="2" t="n"/>
@@ -4935,6 +5308,7 @@
       <c r="H368" s="3" t="n"/>
       <c r="I368" s="3" t="n"/>
       <c r="J368" s="3" t="n"/>
+      <c r="K368" s="3" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="2" t="n"/>
@@ -4947,6 +5321,7 @@
       <c r="H369" s="3" t="n"/>
       <c r="I369" s="3" t="n"/>
       <c r="J369" s="3" t="n"/>
+      <c r="K369" s="3" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="2" t="n"/>
@@ -4959,6 +5334,7 @@
       <c r="H370" s="3" t="n"/>
       <c r="I370" s="3" t="n"/>
       <c r="J370" s="3" t="n"/>
+      <c r="K370" s="3" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="2" t="n"/>
@@ -4971,6 +5347,7 @@
       <c r="H371" s="3" t="n"/>
       <c r="I371" s="3" t="n"/>
       <c r="J371" s="3" t="n"/>
+      <c r="K371" s="3" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="2" t="n"/>
@@ -4983,6 +5360,7 @@
       <c r="H372" s="3" t="n"/>
       <c r="I372" s="3" t="n"/>
       <c r="J372" s="3" t="n"/>
+      <c r="K372" s="3" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="2" t="n"/>
@@ -4995,6 +5373,7 @@
       <c r="H373" s="3" t="n"/>
       <c r="I373" s="3" t="n"/>
       <c r="J373" s="3" t="n"/>
+      <c r="K373" s="3" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="2" t="n"/>
@@ -5007,6 +5386,7 @@
       <c r="H374" s="3" t="n"/>
       <c r="I374" s="3" t="n"/>
       <c r="J374" s="3" t="n"/>
+      <c r="K374" s="3" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="2" t="n"/>
@@ -5019,6 +5399,7 @@
       <c r="H375" s="3" t="n"/>
       <c r="I375" s="3" t="n"/>
       <c r="J375" s="3" t="n"/>
+      <c r="K375" s="3" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="2" t="n"/>
@@ -5031,6 +5412,7 @@
       <c r="H376" s="3" t="n"/>
       <c r="I376" s="3" t="n"/>
       <c r="J376" s="3" t="n"/>
+      <c r="K376" s="3" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="2" t="n"/>
@@ -5043,6 +5425,7 @@
       <c r="H377" s="3" t="n"/>
       <c r="I377" s="3" t="n"/>
       <c r="J377" s="3" t="n"/>
+      <c r="K377" s="3" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="2" t="n"/>
@@ -5055,6 +5438,7 @@
       <c r="H378" s="3" t="n"/>
       <c r="I378" s="3" t="n"/>
       <c r="J378" s="3" t="n"/>
+      <c r="K378" s="3" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="2" t="n"/>
@@ -5067,6 +5451,7 @@
       <c r="H379" s="3" t="n"/>
       <c r="I379" s="3" t="n"/>
       <c r="J379" s="3" t="n"/>
+      <c r="K379" s="3" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="2" t="n"/>
@@ -5079,6 +5464,7 @@
       <c r="H380" s="3" t="n"/>
       <c r="I380" s="3" t="n"/>
       <c r="J380" s="3" t="n"/>
+      <c r="K380" s="3" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="2" t="n"/>
@@ -5091,6 +5477,7 @@
       <c r="H381" s="3" t="n"/>
       <c r="I381" s="3" t="n"/>
       <c r="J381" s="3" t="n"/>
+      <c r="K381" s="3" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="2" t="n"/>
@@ -5103,6 +5490,7 @@
       <c r="H382" s="3" t="n"/>
       <c r="I382" s="3" t="n"/>
       <c r="J382" s="3" t="n"/>
+      <c r="K382" s="3" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="2" t="n"/>
@@ -5115,6 +5503,7 @@
       <c r="H383" s="3" t="n"/>
       <c r="I383" s="3" t="n"/>
       <c r="J383" s="3" t="n"/>
+      <c r="K383" s="3" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="2" t="n"/>
@@ -5127,6 +5516,7 @@
       <c r="H384" s="3" t="n"/>
       <c r="I384" s="3" t="n"/>
       <c r="J384" s="3" t="n"/>
+      <c r="K384" s="3" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="2" t="n"/>
@@ -5139,6 +5529,7 @@
       <c r="H385" s="3" t="n"/>
       <c r="I385" s="3" t="n"/>
       <c r="J385" s="3" t="n"/>
+      <c r="K385" s="3" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="2" t="n"/>
@@ -5151,6 +5542,7 @@
       <c r="H386" s="3" t="n"/>
       <c r="I386" s="3" t="n"/>
       <c r="J386" s="3" t="n"/>
+      <c r="K386" s="3" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="2" t="n"/>
@@ -5163,6 +5555,7 @@
       <c r="H387" s="3" t="n"/>
       <c r="I387" s="3" t="n"/>
       <c r="J387" s="3" t="n"/>
+      <c r="K387" s="3" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="2" t="n"/>
@@ -5175,6 +5568,7 @@
       <c r="H388" s="3" t="n"/>
       <c r="I388" s="3" t="n"/>
       <c r="J388" s="3" t="n"/>
+      <c r="K388" s="3" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="2" t="n"/>
@@ -5187,6 +5581,7 @@
       <c r="H389" s="3" t="n"/>
       <c r="I389" s="3" t="n"/>
       <c r="J389" s="3" t="n"/>
+      <c r="K389" s="3" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="2" t="n"/>
@@ -5199,6 +5594,7 @@
       <c r="H390" s="3" t="n"/>
       <c r="I390" s="3" t="n"/>
       <c r="J390" s="3" t="n"/>
+      <c r="K390" s="3" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="2" t="n"/>
@@ -5211,6 +5607,7 @@
       <c r="H391" s="3" t="n"/>
       <c r="I391" s="3" t="n"/>
       <c r="J391" s="3" t="n"/>
+      <c r="K391" s="3" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="2" t="n"/>
@@ -5223,6 +5620,7 @@
       <c r="H392" s="3" t="n"/>
       <c r="I392" s="3" t="n"/>
       <c r="J392" s="3" t="n"/>
+      <c r="K392" s="3" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="2" t="n"/>
@@ -5235,6 +5633,7 @@
       <c r="H393" s="3" t="n"/>
       <c r="I393" s="3" t="n"/>
       <c r="J393" s="3" t="n"/>
+      <c r="K393" s="3" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="2" t="n"/>
@@ -5247,6 +5646,7 @@
       <c r="H394" s="3" t="n"/>
       <c r="I394" s="3" t="n"/>
       <c r="J394" s="3" t="n"/>
+      <c r="K394" s="3" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="2" t="n"/>
@@ -5259,6 +5659,7 @@
       <c r="H395" s="3" t="n"/>
       <c r="I395" s="3" t="n"/>
       <c r="J395" s="3" t="n"/>
+      <c r="K395" s="3" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="2" t="n"/>
@@ -5271,6 +5672,7 @@
       <c r="H396" s="3" t="n"/>
       <c r="I396" s="3" t="n"/>
       <c r="J396" s="3" t="n"/>
+      <c r="K396" s="3" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="2" t="n"/>
@@ -5283,6 +5685,7 @@
       <c r="H397" s="3" t="n"/>
       <c r="I397" s="3" t="n"/>
       <c r="J397" s="3" t="n"/>
+      <c r="K397" s="3" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="2" t="n"/>
@@ -5295,6 +5698,7 @@
       <c r="H398" s="3" t="n"/>
       <c r="I398" s="3" t="n"/>
       <c r="J398" s="3" t="n"/>
+      <c r="K398" s="3" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="2" t="n"/>
@@ -5307,6 +5711,7 @@
       <c r="H399" s="3" t="n"/>
       <c r="I399" s="3" t="n"/>
       <c r="J399" s="3" t="n"/>
+      <c r="K399" s="3" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="2" t="n"/>
@@ -5319,6 +5724,7 @@
       <c r="H400" s="3" t="n"/>
       <c r="I400" s="3" t="n"/>
       <c r="J400" s="3" t="n"/>
+      <c r="K400" s="3" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="2" t="n"/>
@@ -5331,6 +5737,7 @@
       <c r="H401" s="3" t="n"/>
       <c r="I401" s="3" t="n"/>
       <c r="J401" s="3" t="n"/>
+      <c r="K401" s="3" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="2" t="n"/>
@@ -5343,6 +5750,7 @@
       <c r="H402" s="3" t="n"/>
       <c r="I402" s="3" t="n"/>
       <c r="J402" s="3" t="n"/>
+      <c r="K402" s="3" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="2" t="n"/>
@@ -5355,6 +5763,7 @@
       <c r="H403" s="3" t="n"/>
       <c r="I403" s="3" t="n"/>
       <c r="J403" s="3" t="n"/>
+      <c r="K403" s="3" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="2" t="n"/>
@@ -5367,6 +5776,7 @@
       <c r="H404" s="3" t="n"/>
       <c r="I404" s="3" t="n"/>
       <c r="J404" s="3" t="n"/>
+      <c r="K404" s="3" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="2" t="n"/>
@@ -5379,6 +5789,7 @@
       <c r="H405" s="3" t="n"/>
       <c r="I405" s="3" t="n"/>
       <c r="J405" s="3" t="n"/>
+      <c r="K405" s="3" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="2" t="n"/>
@@ -5391,6 +5802,7 @@
       <c r="H406" s="3" t="n"/>
       <c r="I406" s="3" t="n"/>
       <c r="J406" s="3" t="n"/>
+      <c r="K406" s="3" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="2" t="n"/>
@@ -5403,6 +5815,7 @@
       <c r="H407" s="3" t="n"/>
       <c r="I407" s="3" t="n"/>
       <c r="J407" s="3" t="n"/>
+      <c r="K407" s="3" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="2" t="n"/>
@@ -5415,6 +5828,7 @@
       <c r="H408" s="3" t="n"/>
       <c r="I408" s="3" t="n"/>
       <c r="J408" s="3" t="n"/>
+      <c r="K408" s="3" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="2" t="n"/>
@@ -5427,6 +5841,7 @@
       <c r="H409" s="3" t="n"/>
       <c r="I409" s="3" t="n"/>
       <c r="J409" s="3" t="n"/>
+      <c r="K409" s="3" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="2" t="n"/>
@@ -5439,6 +5854,7 @@
       <c r="H410" s="3" t="n"/>
       <c r="I410" s="3" t="n"/>
       <c r="J410" s="3" t="n"/>
+      <c r="K410" s="3" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="2" t="n"/>
@@ -5451,6 +5867,7 @@
       <c r="H411" s="3" t="n"/>
       <c r="I411" s="3" t="n"/>
       <c r="J411" s="3" t="n"/>
+      <c r="K411" s="3" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="2" t="n"/>
@@ -5463,6 +5880,7 @@
       <c r="H412" s="3" t="n"/>
       <c r="I412" s="3" t="n"/>
       <c r="J412" s="3" t="n"/>
+      <c r="K412" s="3" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="2" t="n"/>
@@ -5475,6 +5893,7 @@
       <c r="H413" s="3" t="n"/>
       <c r="I413" s="3" t="n"/>
       <c r="J413" s="3" t="n"/>
+      <c r="K413" s="3" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="2" t="n"/>
@@ -5487,6 +5906,7 @@
       <c r="H414" s="3" t="n"/>
       <c r="I414" s="3" t="n"/>
       <c r="J414" s="3" t="n"/>
+      <c r="K414" s="3" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="2" t="n"/>
@@ -5499,6 +5919,7 @@
       <c r="H415" s="3" t="n"/>
       <c r="I415" s="3" t="n"/>
       <c r="J415" s="3" t="n"/>
+      <c r="K415" s="3" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="2" t="n"/>
@@ -5511,6 +5932,7 @@
       <c r="H416" s="3" t="n"/>
       <c r="I416" s="3" t="n"/>
       <c r="J416" s="3" t="n"/>
+      <c r="K416" s="3" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="2" t="n"/>
@@ -5523,6 +5945,7 @@
       <c r="H417" s="3" t="n"/>
       <c r="I417" s="3" t="n"/>
       <c r="J417" s="3" t="n"/>
+      <c r="K417" s="3" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="2" t="n"/>
@@ -5535,6 +5958,7 @@
       <c r="H418" s="3" t="n"/>
       <c r="I418" s="3" t="n"/>
       <c r="J418" s="3" t="n"/>
+      <c r="K418" s="3" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="2" t="n"/>
@@ -5547,6 +5971,7 @@
       <c r="H419" s="3" t="n"/>
       <c r="I419" s="3" t="n"/>
       <c r="J419" s="3" t="n"/>
+      <c r="K419" s="3" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="2" t="n"/>
@@ -5559,6 +5984,7 @@
       <c r="H420" s="3" t="n"/>
       <c r="I420" s="3" t="n"/>
       <c r="J420" s="3" t="n"/>
+      <c r="K420" s="3" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="2" t="n"/>
@@ -5571,6 +5997,7 @@
       <c r="H421" s="3" t="n"/>
       <c r="I421" s="3" t="n"/>
       <c r="J421" s="3" t="n"/>
+      <c r="K421" s="3" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="2" t="n"/>
@@ -5583,6 +6010,7 @@
       <c r="H422" s="3" t="n"/>
       <c r="I422" s="3" t="n"/>
       <c r="J422" s="3" t="n"/>
+      <c r="K422" s="3" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="2" t="n"/>
@@ -5595,6 +6023,7 @@
       <c r="H423" s="3" t="n"/>
       <c r="I423" s="3" t="n"/>
       <c r="J423" s="3" t="n"/>
+      <c r="K423" s="3" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="2" t="n"/>
@@ -5607,6 +6036,7 @@
       <c r="H424" s="3" t="n"/>
       <c r="I424" s="3" t="n"/>
       <c r="J424" s="3" t="n"/>
+      <c r="K424" s="3" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="2" t="n"/>
@@ -5619,6 +6049,7 @@
       <c r="H425" s="3" t="n"/>
       <c r="I425" s="3" t="n"/>
       <c r="J425" s="3" t="n"/>
+      <c r="K425" s="3" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="2" t="n"/>
@@ -5631,6 +6062,7 @@
       <c r="H426" s="3" t="n"/>
       <c r="I426" s="3" t="n"/>
       <c r="J426" s="3" t="n"/>
+      <c r="K426" s="3" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="2" t="n"/>
@@ -5643,6 +6075,7 @@
       <c r="H427" s="3" t="n"/>
       <c r="I427" s="3" t="n"/>
       <c r="J427" s="3" t="n"/>
+      <c r="K427" s="3" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="2" t="n"/>
@@ -5655,6 +6088,7 @@
       <c r="H428" s="3" t="n"/>
       <c r="I428" s="3" t="n"/>
       <c r="J428" s="3" t="n"/>
+      <c r="K428" s="3" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="2" t="n"/>
@@ -5667,6 +6101,7 @@
       <c r="H429" s="3" t="n"/>
       <c r="I429" s="3" t="n"/>
       <c r="J429" s="3" t="n"/>
+      <c r="K429" s="3" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="2" t="n"/>
@@ -5679,6 +6114,7 @@
       <c r="H430" s="3" t="n"/>
       <c r="I430" s="3" t="n"/>
       <c r="J430" s="3" t="n"/>
+      <c r="K430" s="3" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="2" t="n"/>
@@ -5691,6 +6127,7 @@
       <c r="H431" s="3" t="n"/>
       <c r="I431" s="3" t="n"/>
       <c r="J431" s="3" t="n"/>
+      <c r="K431" s="3" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="2" t="n"/>
@@ -5703,6 +6140,7 @@
       <c r="H432" s="3" t="n"/>
       <c r="I432" s="3" t="n"/>
       <c r="J432" s="3" t="n"/>
+      <c r="K432" s="3" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="2" t="n"/>
@@ -5715,6 +6153,7 @@
       <c r="H433" s="3" t="n"/>
       <c r="I433" s="3" t="n"/>
       <c r="J433" s="3" t="n"/>
+      <c r="K433" s="3" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="2" t="n"/>
@@ -5727,6 +6166,7 @@
       <c r="H434" s="3" t="n"/>
       <c r="I434" s="3" t="n"/>
       <c r="J434" s="3" t="n"/>
+      <c r="K434" s="3" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="2" t="n"/>
@@ -5739,6 +6179,7 @@
       <c r="H435" s="3" t="n"/>
       <c r="I435" s="3" t="n"/>
       <c r="J435" s="3" t="n"/>
+      <c r="K435" s="3" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="2" t="n"/>
@@ -5751,6 +6192,7 @@
       <c r="H436" s="3" t="n"/>
       <c r="I436" s="3" t="n"/>
       <c r="J436" s="3" t="n"/>
+      <c r="K436" s="3" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="2" t="n"/>
@@ -5763,6 +6205,7 @@
       <c r="H437" s="3" t="n"/>
       <c r="I437" s="3" t="n"/>
       <c r="J437" s="3" t="n"/>
+      <c r="K437" s="3" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="2" t="n"/>
@@ -5775,6 +6218,7 @@
       <c r="H438" s="3" t="n"/>
       <c r="I438" s="3" t="n"/>
       <c r="J438" s="3" t="n"/>
+      <c r="K438" s="3" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="2" t="n"/>
@@ -5787,6 +6231,7 @@
       <c r="H439" s="3" t="n"/>
       <c r="I439" s="3" t="n"/>
       <c r="J439" s="3" t="n"/>
+      <c r="K439" s="3" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="2" t="n"/>
@@ -5799,6 +6244,7 @@
       <c r="H440" s="3" t="n"/>
       <c r="I440" s="3" t="n"/>
       <c r="J440" s="3" t="n"/>
+      <c r="K440" s="3" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="2" t="n"/>
@@ -5811,6 +6257,7 @@
       <c r="H441" s="3" t="n"/>
       <c r="I441" s="3" t="n"/>
       <c r="J441" s="3" t="n"/>
+      <c r="K441" s="3" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="2" t="n"/>
@@ -5823,6 +6270,7 @@
       <c r="H442" s="3" t="n"/>
       <c r="I442" s="3" t="n"/>
       <c r="J442" s="3" t="n"/>
+      <c r="K442" s="3" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="2" t="n"/>
@@ -5835,6 +6283,7 @@
       <c r="H443" s="3" t="n"/>
       <c r="I443" s="3" t="n"/>
       <c r="J443" s="3" t="n"/>
+      <c r="K443" s="3" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="2" t="n"/>
@@ -5847,6 +6296,7 @@
       <c r="H444" s="3" t="n"/>
       <c r="I444" s="3" t="n"/>
       <c r="J444" s="3" t="n"/>
+      <c r="K444" s="3" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="2" t="n"/>
@@ -5859,6 +6309,7 @@
       <c r="H445" s="3" t="n"/>
       <c r="I445" s="3" t="n"/>
       <c r="J445" s="3" t="n"/>
+      <c r="K445" s="3" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="2" t="n"/>
@@ -5871,6 +6322,7 @@
       <c r="H446" s="3" t="n"/>
       <c r="I446" s="3" t="n"/>
       <c r="J446" s="3" t="n"/>
+      <c r="K446" s="3" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="2" t="n"/>
@@ -5883,6 +6335,7 @@
       <c r="H447" s="3" t="n"/>
       <c r="I447" s="3" t="n"/>
       <c r="J447" s="3" t="n"/>
+      <c r="K447" s="3" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="2" t="n"/>
@@ -5895,6 +6348,7 @@
       <c r="H448" s="3" t="n"/>
       <c r="I448" s="3" t="n"/>
       <c r="J448" s="3" t="n"/>
+      <c r="K448" s="3" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="2" t="n"/>
@@ -5907,6 +6361,7 @@
       <c r="H449" s="3" t="n"/>
       <c r="I449" s="3" t="n"/>
       <c r="J449" s="3" t="n"/>
+      <c r="K449" s="3" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="2" t="n"/>
@@ -5919,6 +6374,7 @@
       <c r="H450" s="3" t="n"/>
       <c r="I450" s="3" t="n"/>
       <c r="J450" s="3" t="n"/>
+      <c r="K450" s="3" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="2" t="n"/>
@@ -5931,6 +6387,7 @@
       <c r="H451" s="3" t="n"/>
       <c r="I451" s="3" t="n"/>
       <c r="J451" s="3" t="n"/>
+      <c r="K451" s="3" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="2" t="n"/>
@@ -5943,6 +6400,7 @@
       <c r="H452" s="3" t="n"/>
       <c r="I452" s="3" t="n"/>
       <c r="J452" s="3" t="n"/>
+      <c r="K452" s="3" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="2" t="n"/>
@@ -5955,6 +6413,7 @@
       <c r="H453" s="3" t="n"/>
       <c r="I453" s="3" t="n"/>
       <c r="J453" s="3" t="n"/>
+      <c r="K453" s="3" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="2" t="n"/>
@@ -5967,6 +6426,7 @@
       <c r="H454" s="3" t="n"/>
       <c r="I454" s="3" t="n"/>
       <c r="J454" s="3" t="n"/>
+      <c r="K454" s="3" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="2" t="n"/>
@@ -5979,6 +6439,7 @@
       <c r="H455" s="3" t="n"/>
       <c r="I455" s="3" t="n"/>
       <c r="J455" s="3" t="n"/>
+      <c r="K455" s="3" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="2" t="n"/>
@@ -5991,6 +6452,7 @@
       <c r="H456" s="3" t="n"/>
       <c r="I456" s="3" t="n"/>
       <c r="J456" s="3" t="n"/>
+      <c r="K456" s="3" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="2" t="n"/>
@@ -6003,6 +6465,7 @@
       <c r="H457" s="3" t="n"/>
       <c r="I457" s="3" t="n"/>
       <c r="J457" s="3" t="n"/>
+      <c r="K457" s="3" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="2" t="n"/>
@@ -6015,6 +6478,7 @@
       <c r="H458" s="3" t="n"/>
       <c r="I458" s="3" t="n"/>
       <c r="J458" s="3" t="n"/>
+      <c r="K458" s="3" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="2" t="n"/>
@@ -6027,6 +6491,7 @@
       <c r="H459" s="3" t="n"/>
       <c r="I459" s="3" t="n"/>
       <c r="J459" s="3" t="n"/>
+      <c r="K459" s="3" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="2" t="n"/>
@@ -6039,6 +6504,7 @@
       <c r="H460" s="3" t="n"/>
       <c r="I460" s="3" t="n"/>
       <c r="J460" s="3" t="n"/>
+      <c r="K460" s="3" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="2" t="n"/>
@@ -6051,6 +6517,7 @@
       <c r="H461" s="3" t="n"/>
       <c r="I461" s="3" t="n"/>
       <c r="J461" s="3" t="n"/>
+      <c r="K461" s="3" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="2" t="n"/>
@@ -6063,6 +6530,7 @@
       <c r="H462" s="3" t="n"/>
       <c r="I462" s="3" t="n"/>
       <c r="J462" s="3" t="n"/>
+      <c r="K462" s="3" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="2" t="n"/>
@@ -6075,6 +6543,7 @@
       <c r="H463" s="3" t="n"/>
       <c r="I463" s="3" t="n"/>
       <c r="J463" s="3" t="n"/>
+      <c r="K463" s="3" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="2" t="n"/>
@@ -6087,6 +6556,7 @@
       <c r="H464" s="3" t="n"/>
       <c r="I464" s="3" t="n"/>
       <c r="J464" s="3" t="n"/>
+      <c r="K464" s="3" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="2" t="n"/>
@@ -6099,6 +6569,7 @@
       <c r="H465" s="3" t="n"/>
       <c r="I465" s="3" t="n"/>
       <c r="J465" s="3" t="n"/>
+      <c r="K465" s="3" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="2" t="n"/>
@@ -6111,6 +6582,7 @@
       <c r="H466" s="3" t="n"/>
       <c r="I466" s="3" t="n"/>
       <c r="J466" s="3" t="n"/>
+      <c r="K466" s="3" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="2" t="n"/>
@@ -6123,6 +6595,7 @@
       <c r="H467" s="3" t="n"/>
       <c r="I467" s="3" t="n"/>
       <c r="J467" s="3" t="n"/>
+      <c r="K467" s="3" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="2" t="n"/>
@@ -6135,6 +6608,7 @@
       <c r="H468" s="3" t="n"/>
       <c r="I468" s="3" t="n"/>
       <c r="J468" s="3" t="n"/>
+      <c r="K468" s="3" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="2" t="n"/>
@@ -6147,6 +6621,7 @@
       <c r="H469" s="3" t="n"/>
       <c r="I469" s="3" t="n"/>
       <c r="J469" s="3" t="n"/>
+      <c r="K469" s="3" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="2" t="n"/>
@@ -6159,6 +6634,7 @@
       <c r="H470" s="3" t="n"/>
       <c r="I470" s="3" t="n"/>
       <c r="J470" s="3" t="n"/>
+      <c r="K470" s="3" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="2" t="n"/>
@@ -6171,6 +6647,7 @@
       <c r="H471" s="3" t="n"/>
       <c r="I471" s="3" t="n"/>
       <c r="J471" s="3" t="n"/>
+      <c r="K471" s="3" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="2" t="n"/>
@@ -6183,6 +6660,7 @@
       <c r="H472" s="3" t="n"/>
       <c r="I472" s="3" t="n"/>
       <c r="J472" s="3" t="n"/>
+      <c r="K472" s="3" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="2" t="n"/>
@@ -6195,6 +6673,7 @@
       <c r="H473" s="3" t="n"/>
       <c r="I473" s="3" t="n"/>
       <c r="J473" s="3" t="n"/>
+      <c r="K473" s="3" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="2" t="n"/>
@@ -6207,6 +6686,7 @@
       <c r="H474" s="3" t="n"/>
       <c r="I474" s="3" t="n"/>
       <c r="J474" s="3" t="n"/>
+      <c r="K474" s="3" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="2" t="n"/>
@@ -6219,6 +6699,7 @@
       <c r="H475" s="3" t="n"/>
       <c r="I475" s="3" t="n"/>
       <c r="J475" s="3" t="n"/>
+      <c r="K475" s="3" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="2" t="n"/>
@@ -6231,6 +6712,7 @@
       <c r="H476" s="3" t="n"/>
       <c r="I476" s="3" t="n"/>
       <c r="J476" s="3" t="n"/>
+      <c r="K476" s="3" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="2" t="n"/>
@@ -6243,6 +6725,7 @@
       <c r="H477" s="3" t="n"/>
       <c r="I477" s="3" t="n"/>
       <c r="J477" s="3" t="n"/>
+      <c r="K477" s="3" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="2" t="n"/>
@@ -6255,6 +6738,7 @@
       <c r="H478" s="3" t="n"/>
       <c r="I478" s="3" t="n"/>
       <c r="J478" s="3" t="n"/>
+      <c r="K478" s="3" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="2" t="n"/>
@@ -6267,6 +6751,7 @@
       <c r="H479" s="3" t="n"/>
       <c r="I479" s="3" t="n"/>
       <c r="J479" s="3" t="n"/>
+      <c r="K479" s="3" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="2" t="n"/>
@@ -6279,6 +6764,7 @@
       <c r="H480" s="3" t="n"/>
       <c r="I480" s="3" t="n"/>
       <c r="J480" s="3" t="n"/>
+      <c r="K480" s="3" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="2" t="n"/>
@@ -6291,6 +6777,7 @@
       <c r="H481" s="3" t="n"/>
       <c r="I481" s="3" t="n"/>
       <c r="J481" s="3" t="n"/>
+      <c r="K481" s="3" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="2" t="n"/>
@@ -6303,6 +6790,7 @@
       <c r="H482" s="3" t="n"/>
       <c r="I482" s="3" t="n"/>
       <c r="J482" s="3" t="n"/>
+      <c r="K482" s="3" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="2" t="n"/>
@@ -6315,6 +6803,7 @@
       <c r="H483" s="3" t="n"/>
       <c r="I483" s="3" t="n"/>
       <c r="J483" s="3" t="n"/>
+      <c r="K483" s="3" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="2" t="n"/>
@@ -6327,6 +6816,7 @@
       <c r="H484" s="3" t="n"/>
       <c r="I484" s="3" t="n"/>
       <c r="J484" s="3" t="n"/>
+      <c r="K484" s="3" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="2" t="n"/>
@@ -6339,6 +6829,7 @@
       <c r="H485" s="3" t="n"/>
       <c r="I485" s="3" t="n"/>
       <c r="J485" s="3" t="n"/>
+      <c r="K485" s="3" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="2" t="n"/>
@@ -6351,6 +6842,7 @@
       <c r="H486" s="3" t="n"/>
       <c r="I486" s="3" t="n"/>
       <c r="J486" s="3" t="n"/>
+      <c r="K486" s="3" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="2" t="n"/>
@@ -6363,6 +6855,7 @@
       <c r="H487" s="3" t="n"/>
       <c r="I487" s="3" t="n"/>
       <c r="J487" s="3" t="n"/>
+      <c r="K487" s="3" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="2" t="n"/>
@@ -6375,6 +6868,7 @@
       <c r="H488" s="3" t="n"/>
       <c r="I488" s="3" t="n"/>
       <c r="J488" s="3" t="n"/>
+      <c r="K488" s="3" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="2" t="n"/>
@@ -6387,6 +6881,7 @@
       <c r="H489" s="3" t="n"/>
       <c r="I489" s="3" t="n"/>
       <c r="J489" s="3" t="n"/>
+      <c r="K489" s="3" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="2" t="n"/>
@@ -6399,6 +6894,7 @@
       <c r="H490" s="3" t="n"/>
       <c r="I490" s="3" t="n"/>
       <c r="J490" s="3" t="n"/>
+      <c r="K490" s="3" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="2" t="n"/>
@@ -6411,6 +6907,7 @@
       <c r="H491" s="3" t="n"/>
       <c r="I491" s="3" t="n"/>
       <c r="J491" s="3" t="n"/>
+      <c r="K491" s="3" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="2" t="n"/>
@@ -6423,6 +6920,7 @@
       <c r="H492" s="3" t="n"/>
       <c r="I492" s="3" t="n"/>
       <c r="J492" s="3" t="n"/>
+      <c r="K492" s="3" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="2" t="n"/>
@@ -6435,6 +6933,7 @@
       <c r="H493" s="3" t="n"/>
       <c r="I493" s="3" t="n"/>
       <c r="J493" s="3" t="n"/>
+      <c r="K493" s="3" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="2" t="n"/>
@@ -6447,6 +6946,7 @@
       <c r="H494" s="3" t="n"/>
       <c r="I494" s="3" t="n"/>
       <c r="J494" s="3" t="n"/>
+      <c r="K494" s="3" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="2" t="n"/>
@@ -6459,6 +6959,7 @@
       <c r="H495" s="3" t="n"/>
       <c r="I495" s="3" t="n"/>
       <c r="J495" s="3" t="n"/>
+      <c r="K495" s="3" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="2" t="n"/>
@@ -6471,6 +6972,7 @@
       <c r="H496" s="3" t="n"/>
       <c r="I496" s="3" t="n"/>
       <c r="J496" s="3" t="n"/>
+      <c r="K496" s="3" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="2" t="n"/>
@@ -6483,6 +6985,7 @@
       <c r="H497" s="3" t="n"/>
       <c r="I497" s="3" t="n"/>
       <c r="J497" s="3" t="n"/>
+      <c r="K497" s="3" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="2" t="n"/>
@@ -6495,6 +6998,7 @@
       <c r="H498" s="3" t="n"/>
       <c r="I498" s="3" t="n"/>
       <c r="J498" s="3" t="n"/>
+      <c r="K498" s="3" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="2" t="n"/>
@@ -6507,6 +7011,7 @@
       <c r="H499" s="3" t="n"/>
       <c r="I499" s="3" t="n"/>
       <c r="J499" s="3" t="n"/>
+      <c r="K499" s="3" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="2" t="n"/>
@@ -6519,6 +7024,7 @@
       <c r="H500" s="3" t="n"/>
       <c r="I500" s="3" t="n"/>
       <c r="J500" s="3" t="n"/>
+      <c r="K500" s="3" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="2" t="n"/>
@@ -6531,9 +7037,10 @@
       <c r="H501" s="3" t="n"/>
       <c r="I501" s="3" t="n"/>
       <c r="J501" s="3" t="n"/>
+      <c r="K501" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J501"/>
+  <autoFilter ref="A1:K501"/>
   <dataValidations count="3">
     <dataValidation sqref="D2:D501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valeur invalide" error="La valeur doit être numérique et positive." promptTitle="Dimension" prompt="Saisissez une valeur numérique positive (unité à préciser dans la justification si nécessaire)." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
Use conservative cargo layout screening
</commit_message>
<xml_diff>
--- a/convois_epr2.xlsx
+++ b/convois_epr2.xlsx
@@ -654,7 +654,7 @@
         <v>4.94</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -663,12 +663,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 88.47 m ≤ 154 m; beam 11.35 m ≤ 39 m; draft 4.94 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3000 t DWT, residual DWT 1260 t. Count uses min(geometry bound 3, floor-area bound 6, DWT bound 5); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 88.47 m ≤ 154 m; beam 11.35 m ≤ 39 m; draft 4.94 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3000 t DWT, residual DWT 1840 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 6, DWT bound 5); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Draft 4.94 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 4.94 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold/deck drawing: approximately 57.5 m usable length, 9.0 m width and 8.04 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
@@ -701,7 +701,7 @@
         <v>4.94</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -710,12 +710,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 88.47 m ≤ 154 m; beam 11.35 m ≤ 39 m; draft 4.94 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3000 t DWT, residual DWT 2384 t. Count uses min(geometry bound 4, floor-area bound 7, DWT bound 19); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 88.47 m ≤ 154 m; beam 11.35 m ≤ 39 m; draft 4.94 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3000 t DWT, residual DWT 2846 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 7, DWT bound 19); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Draft 4.94 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 4.94 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold/deck drawing: approximately 57.5 m usable length, 9.0 m width and 8.04 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
@@ -748,7 +748,7 @@
         <v>4.94</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -757,12 +757,12 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 88.47 m ≤ 154 m; beam 11.35 m ≤ 39 m; draft 4.94 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3000 t DWT, residual DWT 2560 t. Count uses min(geometry bound 4, floor-area bound 5, DWT bound 27); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 88.47 m ≤ 154 m; beam 11.35 m ≤ 39 m; draft 4.94 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 2 identical unit(s) theoretical screen maximum; 220 t cargo vs 3000 t DWT, residual DWT 2780 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 5, DWT bound 27); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Draft 4.94 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 4.94 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold/deck drawing: approximately 57.5 m usable length, 9.0 m width and 8.04 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -795,7 +795,7 @@
         <v>5.3</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -804,12 +804,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3300 t DWT, residual DWT 1560 t. Count uses min(geometry bound 3, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3300 t DWT, residual DWT 2140 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
@@ -842,7 +842,7 @@
         <v>5.3</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -851,12 +851,12 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3300 t DWT, residual DWT 2684 t. Count uses min(geometry bound 4, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3300 t DWT, residual DWT 3146 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -889,7 +889,7 @@
         <v>5.3</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -898,12 +898,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3300 t DWT, residual DWT 2860 t. Count uses min(geometry bound 4, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 2 identical unit(s) theoretical screen maximum; 220 t cargo vs 3300 t DWT, residual DWT 3080 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -936,7 +936,7 @@
         <v>5.3</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -945,12 +945,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3300 t DWT, residual DWT 1560 t. Count uses min(geometry bound 3, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3300 t DWT, residual DWT 2140 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
         <v>5.3</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -992,12 +992,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3300 t DWT, residual DWT 2684 t. Count uses min(geometry bound 4, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3300 t DWT, residual DWT 3146 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -1030,7 +1030,7 @@
         <v>5.3</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -1039,12 +1039,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3300 t DWT, residual DWT 2860 t. Count uses min(geometry bound 4, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 2 identical unit(s) theoretical screen maximum; 220 t cargo vs 3300 t DWT, residual DWT 3080 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -1077,7 +1077,7 @@
         <v>5.3</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -1086,12 +1086,12 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3300 t DWT, residual DWT 1560 t. Count uses min(geometry bound 3, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3300 t DWT, residual DWT 2140 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1124,7 +1124,7 @@
         <v>5.3</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -1133,12 +1133,12 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3300 t DWT, residual DWT 2684 t. Count uses min(geometry bound 4, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3300 t DWT, residual DWT 3146 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -1171,7 +1171,7 @@
         <v>5.3</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -1180,12 +1180,12 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3300 t DWT, residual DWT 2860 t. Count uses min(geometry bound 4, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 2 identical unit(s) theoretical screen maximum; 220 t cargo vs 3300 t DWT, residual DWT 3080 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -1218,7 +1218,7 @@
         <v>5.3</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -1227,12 +1227,12 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3300 t DWT, residual DWT 1560 t. Count uses min(geometry bound 3, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3300 t DWT, residual DWT 2140 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
@@ -1265,7 +1265,7 @@
         <v>5.3</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3300 t DWT, residual DWT 2684 t. Count uses min(geometry bound 4, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3300 t DWT, residual DWT 3146 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
@@ -1312,7 +1312,7 @@
         <v>5.3</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1321,12 +1321,12 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3300 t DWT, residual DWT 2860 t. Count uses min(geometry bound 4, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 2 identical unit(s) theoretical screen maximum; 220 t cargo vs 3300 t DWT, residual DWT 3080 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
@@ -1359,7 +1359,7 @@
         <v>5.3</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1368,12 +1368,12 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3300 t DWT, residual DWT 1560 t. Count uses min(geometry bound 3, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3300 t DWT, residual DWT 2140 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 11, DWT bound 5); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
@@ -1406,7 +1406,7 @@
         <v>5.3</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1415,12 +1415,12 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3300 t DWT, residual DWT 2684 t. Count uses min(geometry bound 4, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3300 t DWT, residual DWT 3146 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 13, DWT bound 21); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
@@ -1453,7 +1453,7 @@
         <v>5.3</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1462,12 +1462,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3300 t DWT, residual DWT 2860 t. Count uses min(geometry bound 4, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 86.00 m ≤ 154 m; beam 12.40 m ≤ 39 m; draft 5.30 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 2 identical unit(s) theoretical screen maximum; 220 t cargo vs 3300 t DWT, residual DWT 3080 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 9, DWT bound 30); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.30 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 59.2 m usable length, 10.2 m width and 8.4 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
@@ -1500,7 +1500,7 @@
         <v>5.51</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1509,12 +1509,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3670 t DWT, residual DWT 1930 t. Count uses min(geometry bound 3, floor-area bound 7, DWT bound 6); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3670 t DWT, residual DWT 2510 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 7, DWT bound 6); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 56.6 m usable length, 10.2 m width and 8.13 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
@@ -1547,7 +1547,7 @@
         <v>5.51</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1556,12 +1556,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3670 t DWT, residual DWT 3054 t. Count uses min(geometry bound 4, floor-area bound 8, DWT bound 23); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3670 t DWT, residual DWT 3516 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 8, DWT bound 23); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 56.6 m usable length, 10.2 m width and 8.13 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
@@ -1594,7 +1594,7 @@
         <v>5.51</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1603,12 +1603,12 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3670 t DWT, residual DWT 3230 t. Count uses min(geometry bound 4, floor-area bound 6, DWT bound 33); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 2 identical unit(s) theoretical screen maximum; 220 t cargo vs 3670 t DWT, residual DWT 3450 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 6, DWT bound 33); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 56.6 m usable length, 10.2 m width and 8.13 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
@@ -1641,7 +1641,7 @@
         <v>5.51</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3670 t DWT, residual DWT 1930 t. Count uses min(geometry bound 3, floor-area bound 7, DWT bound 6); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3670 t DWT, residual DWT 2510 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 7, DWT bound 6); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 56.6 m usable length, 10.2 m width and 8.13 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
@@ -1688,7 +1688,7 @@
         <v>5.51</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1697,12 +1697,12 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3670 t DWT, residual DWT 3054 t. Count uses min(geometry bound 4, floor-area bound 8, DWT bound 23); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3670 t DWT, residual DWT 3516 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 8, DWT bound 23); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 56.6 m usable length, 10.2 m width and 8.13 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
@@ -1735,7 +1735,7 @@
         <v>5.51</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -1744,12 +1744,12 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3670 t DWT, residual DWT 3230 t. Count uses min(geometry bound 4, floor-area bound 6, DWT bound 33); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 87.90 m ≤ 154 m; beam 12.80 m ≤ 39 m; draft 5.51 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 2 identical unit(s) theoretical screen maximum; 220 t cargo vs 3670 t DWT, residual DWT 3450 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 6, DWT bound 33); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.51 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 56.6 m usable length, 10.2 m width and 8.13 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
@@ -1782,7 +1782,7 @@
         <v>5.42</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1791,12 +1791,12 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3817 t DWT, residual DWT 2077 t. Count uses min(geometry bound 3, floor-area bound 14, DWT bound 6); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3817 t DWT, residual DWT 2657 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 14, DWT bound 6); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. The uploaded Breb Trader PDF is an older/mismatched sister-sheet labelled Milady/Richelieu; verify the vessel-specific document. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. The uploaded Breb Trader PDF is an older/mismatched sister-sheet labelled Milady/Richelieu; verify the vessel-specific document. Hold drawing: approximately 62.5 m usable length, 10.1 m width and 8.43 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
@@ -1829,7 +1829,7 @@
         <v>5.42</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1838,12 +1838,12 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3817 t DWT, residual DWT 3201 t. Count uses min(geometry bound 4, floor-area bound 16, DWT bound 24); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3817 t DWT, residual DWT 3663 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 16, DWT bound 24); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. The uploaded Breb Trader PDF is an older/mismatched sister-sheet labelled Milady/Richelieu; verify the vessel-specific document. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. The uploaded Breb Trader PDF is an older/mismatched sister-sheet labelled Milady/Richelieu; verify the vessel-specific document. Hold drawing: approximately 62.5 m usable length, 10.1 m width and 8.43 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
@@ -1876,7 +1876,7 @@
         <v>5.42</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1885,12 +1885,12 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3817 t DWT, residual DWT 3377 t. Count uses min(geometry bound 4, floor-area bound 12, DWT bound 34); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 3 identical unit(s) theoretical screen maximum; 330 t cargo vs 3817 t DWT, residual DWT 3487 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 12, DWT bound 34); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. The uploaded Breb Trader PDF is an older/mismatched sister-sheet labelled Milady/Richelieu; verify the vessel-specific document. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. The uploaded Breb Trader PDF is an older/mismatched sister-sheet labelled Milady/Richelieu; verify the vessel-specific document. Hold drawing: approximately 62.5 m usable length, 10.1 m width and 8.43 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
@@ -1923,7 +1923,7 @@
         <v>5.42</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -1932,12 +1932,12 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 3817 t DWT, residual DWT 2077 t. Count uses min(geometry bound 3, floor-area bound 14, DWT bound 6); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 3817 t DWT, residual DWT 2657 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 14, DWT bound 6); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 62.5 m usable length, 10.1 m width and 8.43 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
@@ -1970,7 +1970,7 @@
         <v>5.42</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 4 identical unit(s) theoretical screen maximum; 616 t cargo vs 3817 t DWT, residual DWT 3201 t. Count uses min(geometry bound 4, floor-area bound 16, DWT bound 24); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 3817 t DWT, residual DWT 3663 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 16, DWT bound 24); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 62.5 m usable length, 10.1 m width and 8.43 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -2017,7 +2017,7 @@
         <v>5.42</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -2026,12 +2026,12 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 3817 t DWT, residual DWT 3377 t. Count uses min(geometry bound 4, floor-area bound 12, DWT bound 34); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 88.60 m ≤ 154 m; beam 12.67 m ≤ 39 m; draft 5.42 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 3 identical unit(s) theoretical screen maximum; 330 t cargo vs 3817 t DWT, residual DWT 3487 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 12, DWT bound 34); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 5.42 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 62.5 m usable length, 10.1 m width and 8.43 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K31" s="6" t="inlineStr">
@@ -2064,7 +2064,7 @@
         <v>6.65</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -2073,12 +2073,12 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 6 identical unit(s) theoretical screen maximum; 3480 t cargo vs 4938 t DWT, residual DWT 1458 t. Count uses min(geometry bound 6, floor-area bound 15, DWT bound 8); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 4938 t DWT, residual DWT 3778 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 15, DWT bound 8); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
@@ -2111,7 +2111,7 @@
         <v>6.65</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -2120,12 +2120,12 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 5 identical unit(s) theoretical screen maximum; 770 t cargo vs 4938 t DWT, residual DWT 4168 t. Count uses min(geometry bound 5, floor-area bound 18, DWT bound 32); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 4938 t DWT, residual DWT 4784 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 18, DWT bound 32); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
@@ -2158,7 +2158,7 @@
         <v>6.65</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -2167,12 +2167,12 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 4938 t DWT, residual DWT 4498 t. Count uses min(geometry bound 4, floor-area bound 13, DWT bound 44); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 3 identical unit(s) theoretical screen maximum; 330 t cargo vs 4938 t DWT, residual DWT 4608 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 13, DWT bound 44); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K34" s="6" t="inlineStr">
@@ -2205,7 +2205,7 @@
         <v>6.65</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -2214,12 +2214,12 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 6 identical unit(s) theoretical screen maximum; 3480 t cargo vs 4938 t DWT, residual DWT 1458 t. Count uses min(geometry bound 6, floor-area bound 15, DWT bound 8); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 4938 t DWT, residual DWT 3778 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 15, DWT bound 8); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
@@ -2252,7 +2252,7 @@
         <v>6.65</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -2261,12 +2261,12 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 5 identical unit(s) theoretical screen maximum; 770 t cargo vs 4938 t DWT, residual DWT 4168 t. Count uses min(geometry bound 5, floor-area bound 18, DWT bound 32); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 4938 t DWT, residual DWT 4784 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 18, DWT bound 32); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2299,7 +2299,7 @@
         <v>6.65</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -2308,12 +2308,12 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 4938 t DWT, residual DWT 4498 t. Count uses min(geometry bound 4, floor-area bound 13, DWT bound 44); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 3 identical unit(s) theoretical screen maximum; 330 t cargo vs 4938 t DWT, residual DWT 4608 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 13, DWT bound 44); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -2346,7 +2346,7 @@
         <v>6.65</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2355,12 +2355,12 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 6 identical unit(s) theoretical screen maximum; 3480 t cargo vs 4938 t DWT, residual DWT 1458 t. Count uses min(geometry bound 6, floor-area bound 15, DWT bound 8); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 4938 t DWT, residual DWT 3778 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 15, DWT bound 8); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -2393,7 +2393,7 @@
         <v>6.65</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2402,12 +2402,12 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 5 identical unit(s) theoretical screen maximum; 770 t cargo vs 4938 t DWT, residual DWT 4168 t. Count uses min(geometry bound 5, floor-area bound 18, DWT bound 32); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 4938 t DWT, residual DWT 4784 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 18, DWT bound 32); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -2440,7 +2440,7 @@
         <v>6.65</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -2449,12 +2449,12 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 4938 t DWT, residual DWT 4498 t. Count uses min(geometry bound 4, floor-area bound 13, DWT bound 44); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 3 identical unit(s) theoretical screen maximum; 330 t cargo vs 4938 t DWT, residual DWT 4608 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 13, DWT bound 44); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -2487,7 +2487,7 @@
         <v>6.65</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -2496,12 +2496,12 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 6 identical unit(s) theoretical screen maximum; 3480 t cargo vs 4938 t DWT, residual DWT 1458 t. Count uses min(geometry bound 6, floor-area bound 15, DWT bound 8); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 4938 t DWT, residual DWT 3778 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 15, DWT bound 8); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
@@ -2534,7 +2534,7 @@
         <v>6.65</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -2543,12 +2543,12 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 5 identical unit(s) theoretical screen maximum; 770 t cargo vs 4938 t DWT, residual DWT 4168 t. Count uses min(geometry bound 5, floor-area bound 18, DWT bound 32); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 4938 t DWT, residual DWT 4784 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 18, DWT bound 32); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
@@ -2581,7 +2581,7 @@
         <v>6.65</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -2590,12 +2590,12 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 4938 t DWT, residual DWT 4498 t. Count uses min(geometry bound 4, floor-area bound 13, DWT bound 44); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 89.99 m ≤ 154 m; beam 14.80 m ≤ 39 m; draft 6.65 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 3 identical unit(s) theoretical screen maximum; 330 t cargo vs 4938 t DWT, residual DWT 4608 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 13, DWT bound 44); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.65 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 75.8 m deck length, 11.6 m hold width and 9.23 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K43" s="6" t="inlineStr">
@@ -2628,7 +2628,7 @@
         <v>6.15</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -2637,12 +2637,12 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 6 identical unit(s) theoretical screen maximum; 3480 t cargo vs 5200 t DWT, residual DWT 1720 t. Count uses min(geometry bound 6, floor-area bound 8, DWT bound 8); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 5200 t DWT, residual DWT 4040 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 8, DWT bound 8); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 61.8 m usable length, 11.2 m width and 9.60 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
@@ -2675,7 +2675,7 @@
         <v>6.15</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
@@ -2684,12 +2684,12 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 8 identical unit(s) theoretical screen maximum; 1232 t cargo vs 5200 t DWT, residual DWT 3968 t. Count uses min(geometry bound 8, floor-area bound 10, DWT bound 33); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 5200 t DWT, residual DWT 5046 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 10, DWT bound 33); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 61.8 m usable length, 11.2 m width and 9.60 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -2722,7 +2722,7 @@
         <v>6.15</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2731,12 +2731,12 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 5200 t DWT, residual DWT 4760 t. Count uses min(geometry bound 4, floor-area bound 7, DWT bound 47); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 3 identical unit(s) theoretical screen maximum; 330 t cargo vs 5200 t DWT, residual DWT 4870 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 7, DWT bound 47); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 61.8 m usable length, 11.2 m width and 9.60 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -2769,7 +2769,7 @@
         <v>6.15</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
@@ -2778,12 +2778,12 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 6 identical unit(s) theoretical screen maximum; 3480 t cargo vs 5200 t DWT, residual DWT 1720 t. Count uses min(geometry bound 6, floor-area bound 8, DWT bound 8); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 5200 t DWT, residual DWT 4040 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 8, DWT bound 8); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold drawing: approximately 61.8 m usable length, 11.2 m width and 9.60 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
@@ -2816,7 +2816,7 @@
         <v>6.15</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2825,12 +2825,12 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 8 identical unit(s) theoretical screen maximum; 1232 t cargo vs 5200 t DWT, residual DWT 3968 t. Count uses min(geometry bound 8, floor-area bound 10, DWT bound 33); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 5200 t DWT, residual DWT 5046 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 10, DWT bound 33); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold drawing: approximately 61.8 m usable length, 11.2 m width and 9.60 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
@@ -2863,7 +2863,7 @@
         <v>6.15</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2872,12 +2872,12 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 5200 t DWT, residual DWT 4760 t. Count uses min(geometry bound 4, floor-area bound 7, DWT bound 47); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 99.48 m ≤ 154 m; beam 13.43 m ≤ 39 m; draft 6.15 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 3 identical unit(s) theoretical screen maximum; 330 t cargo vs 5200 t DWT, residual DWT 4870 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 7, DWT bound 47); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.15 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold drawing: approximately 61.8 m usable length, 11.2 m width and 9.60 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -2910,7 +2910,7 @@
         <v>6.5</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2919,12 +2919,12 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 7700 t DWT, residual DWT 1900 t. Count uses min(geometry bound 10, floor-area bound 20, DWT bound 13); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 7700 t DWT, residual DWT 6540 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 20, DWT bound 13); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Two-hold drawing: approximately 51.7 m and 42.7 m hold sections, about 12.0 m width and 9.6–9.9 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
@@ -2957,7 +2957,7 @@
         <v>6.5</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
@@ -2966,12 +2966,12 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 10 identical unit(s) theoretical screen maximum; 1540 t cargo vs 7700 t DWT, residual DWT 6160 t. Count uses min(geometry bound 10, floor-area bound 24, DWT bound 50); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 7700 t DWT, residual DWT 7546 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 24, DWT bound 50); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Two-hold drawing: approximately 51.7 m and 42.7 m hold sections, about 12.0 m width and 9.6–9.9 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
@@ -3004,7 +3004,7 @@
         <v>6.5</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -3013,12 +3013,12 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 6 identical unit(s) theoretical screen maximum; 660 t cargo vs 7700 t DWT, residual DWT 7040 t. Count uses min(geometry bound 6, floor-area bound 18, DWT bound 70); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 7700 t DWT, residual DWT 7260 t. Count uses min(conservative drawing/layout bound 4, floor-area bound 18, DWT bound 70); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Two-hold drawing: approximately 51.7 m and 42.7 m hold sections, about 12.0 m width and 9.6–9.9 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -3051,7 +3051,7 @@
         <v>6.5</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -3060,12 +3060,12 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 7700 t DWT, residual DWT 1900 t. Count uses min(geometry bound 10, floor-area bound 20, DWT bound 13); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 2 identical unit(s) theoretical screen maximum; 1160 t cargo vs 7700 t DWT, residual DWT 6540 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 20, DWT bound 13); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Two-hold drawing: approximately 51.7 m and 42.7 m hold sections, about 12.0 m width and 9.6–9.9 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -3098,7 +3098,7 @@
         <v>6.5</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -3107,12 +3107,12 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 10 identical unit(s) theoretical screen maximum; 1540 t cargo vs 7700 t DWT, residual DWT 6160 t. Count uses min(geometry bound 10, floor-area bound 24, DWT bound 50); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 7700 t DWT, residual DWT 7546 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 24, DWT bound 50); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Two-hold drawing: approximately 51.7 m and 42.7 m hold sections, about 12.0 m width and 9.6–9.9 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr">
@@ -3145,7 +3145,7 @@
         <v>6.5</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
@@ -3154,12 +3154,12 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 6 identical unit(s) theoretical screen maximum; 660 t cargo vs 7700 t DWT, residual DWT 7040 t. Count uses min(geometry bound 6, floor-area bound 18, DWT bound 70); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 125.79 m ≤ 154 m; beam 14.40 m ≤ 39 m; draft 6.50 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 7700 t DWT, residual DWT 7260 t. Count uses min(conservative drawing/layout bound 4, floor-area bound 18, DWT bound 70); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft 6.50 m is below 7 m; verify UKC, tide, squat and port approval against 12 m depth. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Two-hold drawing: approximately 51.7 m and 42.7 m hold sections, about 12.0 m width and 9.6–9.9 m depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K55" s="6" t="inlineStr">
@@ -3192,7 +3192,7 @@
         <v>7</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -3201,12 +3201,12 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 128.45 m ≤ 154 m; beam 16.50 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 8250 t DWT, residual DWT 2450 t. Count uses min(geometry bound 10, floor-area bound 21, DWT bound 14); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 128.45 m ≤ 154 m; beam 16.50 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 8250 t DWT, residual DWT 6510 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 21, DWT bound 14); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Hold/deck drawing: approximately 80.4 m hold length, 13.5 m width and 7.87 m hold depth; CE height requires open/deck loading review. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K56" s="6" t="inlineStr">
@@ -3239,7 +3239,7 @@
         <v>7</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
@@ -3248,12 +3248,12 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 128.45 m ≤ 154 m; beam 16.50 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 10 identical unit(s) theoretical screen maximum; 1540 t cargo vs 8250 t DWT, residual DWT 6710 t. Count uses min(geometry bound 10, floor-area bound 25, DWT bound 53); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 128.45 m ≤ 154 m; beam 16.50 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 1 identical unit(s) theoretical screen maximum; 154 t cargo vs 8250 t DWT, residual DWT 8096 t. Count uses min(conservative drawing/layout bound 1, floor-area bound 25, DWT bound 53); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Hold/deck drawing: approximately 80.4 m hold length, 13.5 m width and 7.87 m hold depth; CE height requires open/deck loading review. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K57" s="6" t="inlineStr">
@@ -3286,7 +3286,7 @@
         <v>7</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -3295,12 +3295,12 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 128.45 m ≤ 154 m; beam 16.50 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 6 identical unit(s) theoretical screen maximum; 660 t cargo vs 8250 t DWT, residual DWT 7590 t. Count uses min(geometry bound 6, floor-area bound 18, DWT bound 75); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 128.45 m ≤ 154 m; beam 16.50 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 4 identical unit(s) theoretical screen maximum; 440 t cargo vs 8250 t DWT, residual DWT 7810 t. Count uses min(conservative drawing/layout bound 4, floor-area bound 18, DWT bound 75); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Hold/deck drawing: approximately 80.4 m hold length, 13.5 m width and 7.87 m hold depth; CE height requires open/deck loading review. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
@@ -3333,7 +3333,7 @@
         <v>7</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -3342,12 +3342,12 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
@@ -3380,7 +3380,7 @@
         <v>7</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -3389,12 +3389,12 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr">
@@ -3427,7 +3427,7 @@
         <v>7</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -3436,12 +3436,12 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
@@ -3474,7 +3474,7 @@
         <v>7</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -3483,12 +3483,12 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
@@ -3521,7 +3521,7 @@
         <v>7</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -3530,12 +3530,12 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr">
@@ -3568,7 +3568,7 @@
         <v>7</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -3577,12 +3577,12 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr">
@@ -3615,7 +3615,7 @@
         <v>7</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -3624,12 +3624,12 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
@@ -3662,7 +3662,7 @@
         <v>7</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -3671,12 +3671,12 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
@@ -3709,7 +3709,7 @@
         <v>7</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -3718,12 +3718,12 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J67" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
@@ -3756,7 +3756,7 @@
         <v>7</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -3765,12 +3765,12 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
@@ -3803,7 +3803,7 @@
         <v>7</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -3812,12 +3812,12 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J69" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
@@ -3850,7 +3850,7 @@
         <v>7</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -3859,12 +3859,12 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
@@ -3897,7 +3897,7 @@
         <v>7</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
@@ -3906,12 +3906,12 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
@@ -3944,7 +3944,7 @@
         <v>7</v>
       </c>
       <c r="G72" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
@@ -3953,12 +3953,12 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -3991,7 +3991,7 @@
         <v>7</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -4000,12 +4000,12 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J73" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -4038,7 +4038,7 @@
         <v>7</v>
       </c>
       <c r="G74" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -4047,12 +4047,12 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr">
@@ -4085,7 +4085,7 @@
         <v>7</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -4094,12 +4094,12 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
@@ -4132,7 +4132,7 @@
         <v>7</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -4141,12 +4141,12 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
@@ -4179,7 +4179,7 @@
         <v>7</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
@@ -4188,12 +4188,12 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J77" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
@@ -4226,7 +4226,7 @@
         <v>7</v>
       </c>
       <c r="G78" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -4235,12 +4235,12 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr">
@@ -4273,7 +4273,7 @@
         <v>7</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -4282,12 +4282,12 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J79" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
@@ -4320,7 +4320,7 @@
         <v>7</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -4329,12 +4329,12 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J80" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
@@ -4367,7 +4367,7 @@
         <v>7</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -4376,12 +4376,12 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J81" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
@@ -4414,7 +4414,7 @@
         <v>7</v>
       </c>
       <c r="G82" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -4423,12 +4423,12 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr">
@@ -4461,7 +4461,7 @@
         <v>7</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -4470,12 +4470,12 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J83" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr">
@@ -4508,7 +4508,7 @@
         <v>7</v>
       </c>
       <c r="G84" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -4517,12 +4517,12 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J84" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
@@ -4555,7 +4555,7 @@
         <v>7</v>
       </c>
       <c r="G85" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -4564,12 +4564,12 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J85" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr">
@@ -4602,7 +4602,7 @@
         <v>7</v>
       </c>
       <c r="G86" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -4611,12 +4611,12 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 10 identical unit(s) theoretical screen maximum; 5800 t cargo vs 9100 t DWT, residual DWT 3300 t. Count uses min(geometry bound 10, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. GV envelope 24.9 × 6.46 × 6.6 m, 580 t each; 3 identical unit(s) theoretical screen maximum; 1740 t cargo vs 9100 t DWT, residual DWT 7360 t. Count uses min(conservative drawing/layout bound 3, floor-area bound 29, DWT bound 15); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J86" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. GV footprint load is about 3.61 t/m²: use a rated tanktop/heavy-cargo position; ordinary deck ratings may be insufficient. Cargo height 6.60 m and hatch/hold clearance require confirmation. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K86" s="6" t="inlineStr">
@@ -4649,7 +4649,7 @@
         <v>7</v>
       </c>
       <c r="G87" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -4658,12 +4658,12 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 12 identical unit(s) theoretical screen maximum; 1848 t cargo vs 9100 t DWT, residual DWT 7252 t. Count uses min(geometry bound 12, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. PP envelope 48 × 2.8 × 3.807 m, 154 t each; 2 identical unit(s) theoretical screen maximum; 308 t cargo vs 9100 t DWT, residual DWT 8792 t. Count uses min(conservative drawing/layout bound 2, floor-area bound 34, DWT bound 59); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J87" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. PP is 48 m long: confirm continuous loading length, hatch arrangement, securing and deck/tanktop rating. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
@@ -4696,7 +4696,7 @@
         <v>7</v>
       </c>
       <c r="G88" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -4705,12 +4705,12 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 12 identical unit(s) theoretical screen maximum; 1320 t cargo vs 9100 t DWT, residual DWT 7780 t. Count uses min(geometry bound 12, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
+          <t>Berth screen PASS: LOA 132.78 m ≤ 154 m; beam 18.85 m ≤ 39 m; draft 7.00 m ≤ 12 m. CE envelope 20 × 9 × 8 m, 110 t each; 5 identical unit(s) theoretical screen maximum; 550 t cargo vs 9100 t DWT, residual DWT 8550 t. Count uses min(conservative drawing/layout bound 5, floor-area bound 26, DWT bound 82); no stacking and no cargo mixing assumed.</t>
         </is>
       </c>
       <c r="J88" s="5" t="inlineStr">
         <is>
-          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
+          <t>Draft is exactly 7.00 m, at the caution threshold; verify UKC, tide, squat and port approval. CE height is 8.00 m: confirm open-deck/hold clearance, hatch opening, securing and stability before acceptance. Main-deck/hold drawing: approximately 112.6 m main-deck length, 18.85 m width and variable 9.04–10.95 m hold depth. DWT is a deadweight screening proxy, not full displacement or stability approval; final loading plan requires owner/naval-architect review.</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">
@@ -4931,13 +4931,13 @@
         <v>3000</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -4977,13 +4977,13 @@
         <v>3300</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -5023,13 +5023,13 @@
         <v>3300</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -5069,13 +5069,13 @@
         <v>3300</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -5115,13 +5115,13 @@
         <v>3300</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -5161,13 +5161,13 @@
         <v>3300</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -5207,13 +5207,13 @@
         <v>3670</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -5253,13 +5253,13 @@
         <v>3670</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -5299,13 +5299,13 @@
         <v>3817</v>
       </c>
       <c r="H10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2" t="n">
         <v>3</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J10" s="2" t="n">
-        <v>4</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -5345,13 +5345,13 @@
         <v>3817</v>
       </c>
       <c r="H11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="2" t="n">
         <v>3</v>
-      </c>
-      <c r="I11" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J11" s="2" t="n">
-        <v>4</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -5391,13 +5391,13 @@
         <v>4938</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -5437,13 +5437,13 @@
         <v>4938</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -5483,13 +5483,13 @@
         <v>4938</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -5529,13 +5529,13 @@
         <v>4938</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -5575,13 +5575,13 @@
         <v>5200</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -5621,13 +5621,13 @@
         <v>5200</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
@@ -5667,13 +5667,13 @@
         <v>7700</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
@@ -5713,13 +5713,13 @@
         <v>7700</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
@@ -5759,13 +5759,13 @@
         <v>8250</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
@@ -5805,13 +5805,13 @@
         <v>9100</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
@@ -5851,13 +5851,13 @@
         <v>9100</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
@@ -5897,13 +5897,13 @@
         <v>9100</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -5943,13 +5943,13 @@
         <v>9100</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -5989,13 +5989,13 @@
         <v>9100</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -6035,13 +6035,13 @@
         <v>9100</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -6081,13 +6081,13 @@
         <v>9100</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
@@ -6127,13 +6127,13 @@
         <v>9100</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -6173,13 +6173,13 @@
         <v>9100</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -6219,13 +6219,13 @@
         <v>9100</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
@@ -6548,7 +6548,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Theoretical count = minimum of geometry upper bound, available floor-area bound and DWT/mass bound. No stacking is assumed.</t>
+          <t>Theoretical count = minimum of a conservative hold/main-deck drawing bound, available floor-area bound and DWT/mass bound. No stacking is assumed.</t>
         </is>
       </c>
     </row>
@@ -6560,7 +6560,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Geometry uses overall LOA and beam as a screening upper bound; it is not a substitute for a final stowage plan or hatch/hold drawing.</t>
+          <t>The drawing bounds are approximate screening values; final stowage still requires vessel-specific hatch, access, securing and stability approval.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document second-filter rules in workbooks
</commit_message>
<xml_diff>
--- a/convois_epr2.xlsx
+++ b/convois_epr2.xlsx
@@ -89,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -107,12 +107,21 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -159,6 +168,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6911,11 +6922,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -7238,9 +7249,79 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>Second filter rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>1. Prefer a single-decker with no tween/intermediate deck.</t>
+        </is>
+      </c>
+      <c r="B32" s="23" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2. If a tween deck exists, cargo must clear it or the deck must be removed/landed ashore.</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>3. Hatch opening and hold access must accept the cargo length and allow loading/unloading.</t>
+        </is>
+      </c>
+      <c r="B34" s="23" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>4. Cargo footprint must stay within the deck/tanktop rating; GV is about 3.61 t/m².</t>
+        </is>
+      </c>
+      <c r="B35" s="23" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>5. After deck, opening and load checks pass, choose the lowest published fuel consumption.</t>
+        </is>
+      </c>
+      <c r="B36" s="23" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>6. Draft above 7 m is a caution; maximum available depth is 12 m.</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>7. Missing deck/opening/fuel data means conditional, not final approval.</t>
+        </is>
+      </c>
+      <c r="B38" s="23" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="8">
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A33:B33"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId1"/>

</xml_diff>

<commit_message>
Make Pride loading status conditional
</commit_message>
<xml_diff>
--- a/convois_epr2.xlsx
+++ b/convois_epr2.xlsx
@@ -89,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -116,12 +116,18 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -170,6 +176,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -719,12 +728,12 @@
       </c>
       <c r="J2" s="12" t="inlineStr">
         <is>
-          <t>SELECTED: single deck; no tween deck; 4.5 t/day.</t>
+          <t>CONDITIONAL: hold about 9.00×8.04 m fits cargo only; full GV convoy is about 7.78 m high (0.26 m clearance); gearless vessel needs shore lifting; confirm hatch opening and crane.</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Check hatch clearance, securing, stability and UKC.</t>
+          <t>Caution: full convoy clearance is only about 0.26 m; confirm hatch, trailer and shore crane.</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -771,12 +780,12 @@
       </c>
       <c r="J3" s="12" t="inlineStr">
         <is>
-          <t>SELECTED: single deck; no tween deck; 4.5 t/day.</t>
+          <t>CONDITIONAL: hold about 9.00×8.04 m fits cargo only; full GV convoy is about 7.78 m high (0.26 m clearance); gearless vessel needs shore lifting; confirm hatch opening and crane.</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Check hatch clearance, securing, stability and UKC.</t>
+          <t>Caution: full convoy clearance is only about 0.26 m; confirm hatch, trailer and shore crane.</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -823,12 +832,12 @@
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>SELECTED: single deck; no tween deck; 4.5 t/day.</t>
+          <t>CONDITIONAL: hold about 9.00×8.04 m fits cargo only; full GV convoy is about 7.78 m high (0.26 m clearance); gearless vessel needs shore lifting; confirm hatch opening and crane.</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Check hatch clearance, securing, stability and UKC.</t>
+          <t>Caution: full convoy clearance is only about 0.26 m; confirm hatch, trailer and shore crane.</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -5397,51 +5406,51 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="n">
+      <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Pride</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>Conventional</t>
-        </is>
-      </c>
-      <c r="D2" s="14" t="n">
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Conventional</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="n">
         <v>88.47</v>
       </c>
-      <c r="E2" s="14" t="n">
+      <c r="E2" s="17" t="n">
         <v>11.35</v>
       </c>
-      <c r="F2" s="14" t="n">
+      <c r="F2" s="17" t="n">
         <v>4.94</v>
       </c>
-      <c r="G2" s="13" t="n">
+      <c r="G2" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="H2" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="I2" s="13" t="n">
+      <c r="H2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="K2" s="13" t="inlineStr">
+      <c r="J2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
         <is>
           <t>PASS (154 m / 39 m / 12 m)</t>
         </is>
       </c>
-      <c r="L2" s="15" t="inlineStr">
-        <is>
-          <t>SELECTED: single deck; no tween deck; 4.5 t/day.</t>
-        </is>
-      </c>
-      <c r="M2" s="16" t="inlineStr">
+      <c r="L2" s="18" t="inlineStr">
+        <is>
+          <t>CONDITIONAL: hold about 9.00×8.04 m fits cargo only; full GV convoy is about 7.78 m high (0.26 m clearance); gearless vessel needs shore lifting; confirm hatch opening and crane.</t>
+        </is>
+      </c>
+      <c r="M2" s="19" t="inlineStr">
         <is>
           <t>https://github.com/swatheeshkaran-max/edf-dechargement-colis/blob/main/briese_pdf/pride.pdf</t>
         </is>
@@ -6922,7 +6931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -7257,7 +7266,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="24" t="inlineStr">
         <is>
           <t>1. Prefer a single-decker with no tween/intermediate deck.</t>
         </is>
@@ -7265,7 +7274,7 @@
       <c r="B32" s="23" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="24" t="inlineStr">
         <is>
           <t>2. If a tween deck exists, cargo must clear it or the deck must be removed/landed ashore.</t>
         </is>
@@ -7273,7 +7282,7 @@
       <c r="B33" s="23" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="24" t="inlineStr">
         <is>
           <t>3. Hatch opening and hold access must accept the cargo length and allow loading/unloading.</t>
         </is>
@@ -7281,7 +7290,7 @@
       <c r="B34" s="23" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="24" t="inlineStr">
         <is>
           <t>4. Cargo footprint must stay within the deck/tanktop rating; GV is about 3.61 t/m².</t>
         </is>
@@ -7289,7 +7298,7 @@
       <c r="B35" s="23" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="24" t="inlineStr">
         <is>
           <t>5. After deck, opening and load checks pass, choose the lowest published fuel consumption.</t>
         </is>
@@ -7297,7 +7306,7 @@
       <c r="B36" s="23" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="24" t="inlineStr">
         <is>
           <t>6. Draft above 7 m is a caution; maximum available depth is 12 m.</t>
         </is>
@@ -7305,12 +7314,24 @@
       <c r="B37" s="23" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="24" t="inlineStr">
         <is>
           <t>7. Missing deck/opening/fuel data means conditional, not final approval.</t>
         </is>
       </c>
       <c r="B38" s="23" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>Loading check note</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>For a complete convoy, use convoy width/height and lifting method, not cargo dimensions alone.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
Apply hold-width clearance to Pride CE loading
</commit_message>
<xml_diff>
--- a/convois_epr2.xlsx
+++ b/convois_epr2.xlsx
@@ -728,7 +728,7 @@
       </c>
       <c r="J2" s="12" t="inlineStr">
         <is>
-          <t>CONDITIONAL: hold about 9.00×8.04 m fits cargo only; full GV convoy is about 7.78 m high (0.26 m clearance); gearless vessel needs shore lifting; confirm hatch opening and crane.</t>
+          <t>CONDITIONAL: width clearance is adequate for cargo-only loading; full convoy height, hatch opening and shore crane still need confirmation.</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="J3" s="12" t="inlineStr">
         <is>
-          <t>CONDITIONAL: hold about 9.00×8.04 m fits cargo only; full GV convoy is about 7.78 m high (0.26 m clearance); gearless vessel needs shore lifting; confirm hatch opening and crane.</t>
+          <t>CONDITIONAL: width clearance is adequate for cargo-only loading; full convoy height, hatch opening and shore crane still need confirmation.</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -818,7 +818,7 @@
         <v>4.94</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -827,17 +827,17 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>1st filter PASS: 88.47×11.35×4.94 m; 2 CE; berth 154×39×12 m.</t>
+          <t>1st filter PASS: 88.47×11.35×4.94 m; 0 CE; berth 154×39×12 m.</t>
         </is>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>CONDITIONAL: hold about 9.00×8.04 m fits cargo only; full GV convoy is about 7.78 m high (0.26 m clearance); gearless vessel needs shore lifting; confirm hatch opening and crane.</t>
+          <t>HOLD: CE width 9.00 m = hold width 9.00 m; zero clearance.</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Caution: full convoy clearance is only about 0.26 m; confirm hatch, trailer and shore crane.</t>
+          <t>Need at least 0.50 m clearance each side; CE not accepted in Pride.</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -5438,7 +5438,7 @@
         <v>1</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
@@ -5447,7 +5447,7 @@
       </c>
       <c r="L2" s="18" t="inlineStr">
         <is>
-          <t>CONDITIONAL: hold about 9.00×8.04 m fits cargo only; full GV convoy is about 7.78 m high (0.26 m clearance); gearless vessel needs shore lifting; confirm hatch opening and crane.</t>
+          <t>CONDITIONAL: GV/PP width clearance is adequate; CE 9.00 m equals the 9.00 m hold width, so CE is rejected. Full convoy/hatch/crane check remains.</t>
         </is>
       </c>
       <c r="M2" s="19" t="inlineStr">
@@ -6931,7 +6931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -7330,6 +7330,18 @@
       <c r="B40" s="21" t="inlineStr">
         <is>
           <t>For a complete convoy, use convoy width/height and lifting method, not cargo dimensions alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>Clearance rule</t>
+        </is>
+      </c>
+      <c r="B42" s="21" t="inlineStr">
+        <is>
+          <t>Require cargo width + 1.00 m minimum (0.50 m each side) inside the clear hold/hatch width; equal widths fail.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document ECO sister-vessel tie
</commit_message>
<xml_diff>
--- a/convois_epr2.xlsx
+++ b/convois_epr2.xlsx
@@ -3848,7 +3848,7 @@
       </c>
       <c r="J62" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="J63" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K63" s="5" t="inlineStr">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="J64" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr">
@@ -4004,7 +4004,7 @@
       </c>
       <c r="J65" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K65" s="5" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="J66" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K66" s="5" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="J67" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K67" s="5" t="inlineStr">
@@ -4160,7 +4160,7 @@
       </c>
       <c r="J68" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K68" s="5" t="inlineStr">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="J69" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K69" s="5" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="J70" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K70" s="5" t="inlineStr">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="J71" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K71" s="5" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J72" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K72" s="5" t="inlineStr">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="J73" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K73" s="5" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="J74" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K74" s="5" t="inlineStr">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="J75" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K75" s="5" t="inlineStr">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="J76" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K76" s="5" t="inlineStr">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="J77" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K77" s="5" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="J78" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K78" s="5" t="inlineStr">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="J79" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K79" s="5" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="J80" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K80" s="5" t="inlineStr">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="J81" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K81" s="5" t="inlineStr">
@@ -4888,7 +4888,7 @@
       </c>
       <c r="J82" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K82" s="5" t="inlineStr">
@@ -4940,7 +4940,7 @@
       </c>
       <c r="J83" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K83" s="5" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="J84" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K84" s="5" t="inlineStr">
@@ -5044,7 +5044,7 @@
       </c>
       <c r="J85" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K85" s="5" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="J86" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K86" s="5" t="inlineStr">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="J87" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K87" s="5" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J88" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="K88" s="5" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="L22" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
@@ -6518,7 +6518,7 @@
       </c>
       <c r="L23" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="M23" s="6" t="inlineStr">
@@ -6569,7 +6569,7 @@
       </c>
       <c r="L24" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="M24" s="6" t="inlineStr">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="L25" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
@@ -6671,7 +6671,7 @@
       </c>
       <c r="L26" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="M26" s="6" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="L27" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="M27" s="6" t="inlineStr">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="L28" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="M28" s="6" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="L29" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="M29" s="6" t="inlineStr">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="L30" s="12" t="inlineStr">
         <is>
-          <t>Not shortlisted in 2nd filter.</t>
+          <t>TIE: same ECO specification as Titan; 3 tween heights, 4.0 t/m² tween rating, 7.6 t/day. No second-filter failure.</t>
         </is>
       </c>
       <c r="M30" s="6" t="inlineStr">
@@ -6931,7 +6931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -7342,6 +7342,18 @@
       <c r="B42" s="21" t="inlineStr">
         <is>
           <t>Require cargo width + 1.00 m minimum (0.50 m each side) inside the clear hold/hatch width; equal widths fail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>ECO group note</t>
+        </is>
+      </c>
+      <c r="B44" s="21" t="inlineStr">
+        <is>
+          <t>ECO Titan was one representative only; ECO Trust and the other ECO vessels tie on the published second-filter data.</t>
         </is>
       </c>
     </row>

</xml_diff>